<commit_message>
Enhance report generation workflow and sidebar UX
</commit_message>
<xml_diff>
--- a/config/Framework_Intelligence.xlsx
+++ b/config/Framework_Intelligence.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Shubham.baranwal\Downloads\Company_Report_Generator\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5676CEDE-2899-4456-B4C9-DA8899D8B8ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{481A9BF5-BDDB-4273-97B5-B72E54F5391B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -841,25 +841,6 @@
     <t>Analyze the company using the Porter's Five Forces framework. Competitive analysis with Low/Medium/High ratings and one-line justification for each force (Do not mention justification work, instead mention the justification point directly). Includes overall industry attractiveness Focus on strategic, evidence-backed insights derived from public information. Keep the analysis concise, executive-ready, and actionable.</t>
   </si>
   <si>
-    <t>Analyze {Company_Name} using SWOT Analysis.
-Objective:
-2–3 concise, crisp, evidence-backed points for quadrant: Strengths, Weaknesses, Opportunities, Threats
-Instructions:
-- Use reliable publicly available information and recent business context.
-- Focus on strategic insights rather than generic statements.
-- Keep each point concise and evidence-backed.
-- Avoid unsupported speculation.
-- Follow this representation: Four-quadrant color-coded matrix with 2-3 bullet points.
-- Conclude with a one-line executive takeaway highlighting the most Important implications.
-- Output MUST be in GitHub Markdown.
-- DO NOT generate HTML.
-- DO NOT use &lt;table&gt;, &lt;div&gt;, or CSS.
-- Use Markdown tables.
-- Use Markdown headings.
-- Never wrap output in code fences.
-- End with crisp short Executive Takeaway.</t>
-  </si>
-  <si>
     <t xml:space="preserve">Analyze {Company_Name} using the PESTLE framework.
 Objective:
 Political, Economic, Social, Technological, Environmental, and Legal. Concise pointer under each point
@@ -869,7 +850,7 @@
 - Keep each point concise and evidence-backed.
 - Avoid unsupported speculation.
 - Follow this representation: 6 cards with details within.
-- Conclude with a one-two line crisp short executive takeaway highlighting the most Important implications.
+- Conclude with a 3 to 4 line crisp short executive takeaway highlighting the most Important implications.
 - Output MUST be in GitHub Markdown.
 - DO NOT generate HTML.
 - DO NOT use &lt;table&gt;, &lt;div&gt;, or CSS.
@@ -880,6 +861,564 @@
 </t>
   </si>
   <si>
+    <t xml:space="preserve">Analyze {Company_Name} using the ESG Assessment framework.
+Objective:
+Environmental initiatives, social responsibility, governance practices, Public ESG rating
+Instructions:
+- Use reliable publicly available information and recent business context.
+- Focus on strategic insights rather than generic statements.
+- Keep each point concise and evidence-backed.
+- Avoid unsupported speculation.
+- Follow this representation: ESG cards with Maturity status.
+- Conclude with a 3 to 4 line crisp short executive takeaway highlighting the most Important implications.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Analyze {Company_Name} using the Partnership Ecosystem framework.
+Objective:
+Evaluate the company using the principles of this framework.
+Instructions:
+- Use reliable publicly available information and recent business context.
+- Focus on strategic insights rather than generic statements.
+- Keep each point concise and evidence-backed.
+- Avoid unsupported speculation.
+- Follow this representation: Executive summary.
+- Conclude with a 3 to 4 line crisp short executive takeaway highlighting the most Important implications.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Analyze {Company_Name} using the Innovation Assessment framework.
+Objective:
+R&amp;D focus, patents, AI investments, innovation culture, product launches
+Instructions:
+- Use reliable publicly available information and recent business context.
+- Focus on strategic insights rather than generic statements.
+- Keep each point concise and evidence-backed.
+- Avoid unsupported speculation.
+- Follow this representation: Concise points on innovation initiatives.
+- Conclude with a 3 to 4 line crisp short executive takeaway highlighting the most Important implications.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Analyze {Company_Name} using the GE-McKinsey Nine-Box Matrix framework.
+Objective:
+Business unit attractiveness vs competitive strength (high-level assessment)
+Instructions:
+- Use reliable publicly available information and recent business context.
+- Focus on strategic insights rather than generic statements.
+- Keep each point concise and evidence-backed.
+- Avoid unsupported speculation.
+- Follow this representation: 3×3 matrix with highlighted business units.
+- Conclude with a 3 to 4 line crisp short executive takeaway highlighting the most Important implications.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Analyze {Company_Name} using the Strategic Partnership Opportunities framework.
+Objective:
+Highlights where company partners strategically to create competitive advantage. Contains Strategic objective, Key partnership categories, Major partners, Partnership model, Value to Company, Value to Partner, Competitive advantage created, Risk factors, and Overall Strategic Partnership Maturity
+Instructions:
+- Use reliable publicly available information and recent business context.
+- Focus on strategic insights rather than generic statements.
+- Keep each point concise and evidence-backed.
+- Avoid unsupported speculation.
+- Follow this representation: Concise pointers for each points in tabular form with partnership maturity score.
+- Conclude with a 3 to 4 line crisp short executive takeaway highlighting the most Important implications.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Analyze {Company_Name} using the Sustainability Assessment framework.
+Objective:
+Overall digital maturity level, cloud adoption, AI adoption, engineering maturity, data capabilities, security posture. Tech stack details visible only for Technical Leads
+Instructions:
+- Use reliable publicly available information and recent business context.
+- Focus on strategic insights rather than generic statements.
+- Keep each point concise and evidence-backed.
+- Avoid unsupported speculation.
+- Follow this representation: Concise pointers under each of economic, innovation, etc along with overall sustainability score (out of 5).
+- Conclude with a 3 to 4 line crisp short executive takeaway highlighting the most Important implications.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Analyze {Company_Name} using the McKinsey 7S framework framework.
+Objective:
+Assessment of company on 7 Elements: Strategy, Structure, system, Shared values, staff, skill and style; with a pointer on current state for each element and assessment of each pointer as Strong/average/weak
+Instructions:
+- Use reliable publicly available information and recent business context.
+- Focus on strategic insights rather than generic statements.
+- Keep each point concise and evidence-backed.
+- Avoid unsupported speculation.
+- Follow this representation: 7 cards for each elements with a concise point within each card with assessment/maturity of company on each element. With overall score.
+- Conclude with a 3 to 4 line crisp short executive takeaway highlighting the most Important implications.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Analyze {Company_Name} using the Greiner Growth Model framework.
+Objective:
+Organization evolution through 6 growth phases, current position of company in 6 growth phases, status of each phases for the company, current growth challenges (3-4 key challenges and business impact)
+Instructions:
+- Use reliable publicly available information and recent business context.
+- Focus on strategic insights rather than generic statements.
+- Keep each point concise and evidence-backed.
+- Avoid unsupported speculation.
+- Follow this representation: Company position in Greiner's model curve, evolution through each phase (concise 1 sensentce on each phase) with status as Completed/Current stage/Emerging/future.
+- Conclude with a 3 to 4 line crisp short executive takeaway highlighting the most Important implications.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Analyze {Company_Name} using the Hoshin Kanri framework.
+Objective:
+Framework shows strategy deployment, how a company's vision cascades into execution and how execution feeds back into continuous improvement.
+Instructions:
+- Use reliable publicly available information and recent business context.
+- Focus on strategic insights rather than generic statements.
+- Keep each point concise and evidence-backed.
+- Avoid unsupported speculation.
+- Follow this representation: Hoshin Kanri Strategy Cascade with True north, Breakthrough Goals, Annual priorities, Strategic initiatives, KPIs, and Review.
+- Conclude with a 3 to 4 line crisp short executive takeaway highlighting the most Important implications.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Analyze {Company_Name} using the McKinsey's 3 Horizons of Growth framework.
+Objective:
+3 Horizon snapshot of the company including their focus, initiatives and strategic maturity. Along with horizon wise evaluation including objective, initiatives, assessment and overall 3 horizon score
+Instructions:
+- Use reliable publicly available information and recent business context.
+- Focus on strategic insights rather than generic statements.
+- Keep each point concise and evidence-backed.
+- Avoid unsupported speculation.
+- Follow this representation: 3 horizon snapshot and horizon wise evaluation , 3-4 concise pointer within each horizon and Assessment of each horizon, along with overall score.
+- Conclude with a 3 to 4 line crisp short executive takeaway highlighting the most Important implications.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Analyze {Company_Name} using the TOWS Matrix framework.
+Objective:
+Putting SWOT analysis to action, combines Internal (Strength and weakness) and External (Opportunity and threats) factors to derive strategic actions/plans
+Instructions:
+- Use reliable publicly available information and recent business context.
+- Focus on strategic insights rather than generic statements.
+- Keep each point concise and evidence-backed.
+- Avoid unsupported speculation.
+- Follow this representation: 4 quadrant colour-coded matrix with 2-3 concise points in each quadrant of TOWS matrix.
+- Conclude with a 3 to 4 line crisp short executive takeaway highlighting the most Important implications.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Analyze {Company_Name} using the VRIO Framework framework.
+Objective:
+Used to evaluate a company's internal resources and capabilities and its ability to sustain competitive advantage. Contains strategic resource/capability VRIO Assessment Matrix along with executive score card of each of VRIO elements
+Instructions:
+- Use reliable publicly available information and recent business context.
+- Focus on strategic insights rather than generic statements.
+- Keep each point concise and evidence-backed.
+- Avoid unsupported speculation.
+- Follow this representation: Strategic Resource/Capability assessment matrix on VRIO with competitive implications, and 4 quadrants with executive score under each of Value, Rarity, Imitability, and Organization elements.
+- Conclude with a 3 to 4 line crisp short executive takeaway highlighting the most Important implications.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Analyze {Company_Name} using the Porter's Diamond Model framework.
+Objective:
+Utilized to evaluate domain or industry the company belongs to. For example, it will better evaluate insurance/healthcare domain than individual company in it
+Instructions:
+- Use reliable publicly available information and recent business context.
+- Focus on strategic insights rather than generic statements.
+- Keep each point concise and evidence-backed.
+- Avoid unsupported speculation.
+- Follow this representation: Four cards for each of the diamonds in the framework.
+- Conclude with a 3 to 4 line crisp short executive takeaway highlighting the most Important implications.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Analyze {Company_Name} using the Strategic Group Mapping framework.
+Objective:
+Overall position of company, with a 2x2 strategic group map, current strategic groups, closest competitiors, key differentiators and executive insights
+Instructions:
+- Use reliable publicly available information and recent business context.
+- Focus on strategic insights rather than generic statements.
+- Keep each point concise and evidence-backed.
+- Avoid unsupported speculation.
+- Follow this representation: 1-line summary with score with a scatter plot for 2x2 map, strategic group cards with competitors, 1-line insights.
+- Conclude with a 3 to 4 line crisp short executive takeaway highlighting the most Important implications.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Analyze {Company_Name} using the Bowman's Strategy Clock framework.
+Objective:
+Maps company's competitive position on 2 axes,  price vs perceived value/differentiation  - into 8 distinct positions (low price/low value, low price, hybrid, differentiation, focused differentiation, and three "doomed" high-price/low-value zones)
+Instructions:
+- Use reliable publicly available information and recent business context.
+- Focus on strategic insights rather than generic statements.
+- Keep each point concise and evidence-backed.
+- Avoid unsupported speculation.
+- Follow this representation: Price vs Perceived value chart with 8 positions.
+- Conclude with a 3 to 4 line crisp short executive takeaway highlighting the most Important implications.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Analyze {Company_Name} using the Strategy Diamond framework.
+Objective:
+A strategy model that structures and challenges a company's strategic plan to make it more comprehensive and clear. Contains 5 elements Arenas, Vehicles, Differentiators, Staging and Pacing, and Economic logic
+Instructions:
+- Use reliable publicly available information and recent business context.
+- Focus on strategic insights rather than generic statements.
+- Keep each point concise and evidence-backed.
+- Avoid unsupported speculation.
+- Follow this representation: 5 cards for each element arranged in diamond shape or + shape.
+- Conclude with a 3 to 4 line crisp short executive takeaway highlighting the most Important implications.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Analyze {Company_Name} using the Three C's Framework (Company, Customer, Competitor) framework.
+Objective:
+Concise line under each of  Company, Customer, Competitor, Competitive edge, and Strategic insight with respect to the company
+Instructions:
+- Use reliable publicly available information and recent business context.
+- Focus on strategic insights rather than generic statements.
+- Keep each point concise and evidence-backed.
+- Avoid unsupported speculation.
+- Follow this representation: 5 cards placed in a triagular shape with Company, customers and competitor at its edge, two card with Competitive edge and Strategic insight below them.
+- Conclude with a 3 to 4 line crisp short executive takeaway highlighting the most Important implications.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Analyze {Company_Name} using the VMOST Framework framework.
+Objective:
+It showcases if a company's Vision, Mission, Objectives, Strategy, and Tactics are aligned to execute its long-term business goals. It shows concise view of strategic direction and execution maturity
+Instructions:
+- Use reliable publicly available information and recent business context.
+- Focus on strategic insights rather than generic statements.
+- Keep each point concise and evidence-backed.
+- Avoid unsupported speculation.
+- Follow this representation: VMOST snapshot with 5 components, 1 line assessment of each component and Overall alignment towards its vission and mission.
+- Conclude with a 3 to 4 line crisp short executive takeaway highlighting the most Important implications.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Analyze {Company_Name} using the SOAR Analysis framework.
+Objective:
+Showcases company's strengths, opportunities, aspirations and results (performance metrics) and how well is it performing
+Instructions:
+- Use reliable publicly available information and recent business context.
+- Focus on strategic insights rather than generic statements.
+- Keep each point concise and evidence-backed.
+- Avoid unsupported speculation.
+- Follow this representation: 4 cards with concise line under each of Strengths, opportunities, aspirations and results.
+- Conclude with a 3 to 4 line crisp short executive takeaway highlighting the most Important implications.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Analyze {Company_Name} using the NOISE Analysis framework.
+Objective:
+It evaluates company on 5 core elements i.e. needs, opportunities, improvements, strengths, and exceptions. It provides comprehensive business overview and helps create solution oriented action plan
+Instructions:
+- Use reliable publicly available information and recent business context.
+- Focus on strategic insights rather than generic statements.
+- Keep each point concise and evidence-backed.
+- Avoid unsupported speculation.
+- Follow this representation: Executive summary along with 5 cards for core elements Needs, opportunity, improvments, strengths and exceptions with  performance in each of them.
+- Conclude with a 3 to 4 line crisp short executive takeaway highlighting the most Important implications.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Analyze {Company_Name} using the ADL Matrix framework.
+Objective:
+Evaluate company on Industry maturity stage (Embryonic, Growth, Mature, and Aging) and Competitive position (Dominant, Strong, Favorable, Tenable, and Weak)
+Instructions:
+- Use reliable publicly available information and recent business context.
+- Focus on strategic insights rather than generic statements.
+- Keep each point concise and evidence-backed.
+- Avoid unsupported speculation.
+- Follow this representation: Company position in 4x5 matrix of Industry Maturity vs Competitve position, explanation why at certain Industry maturity and competitve position backed with evidence and strategic implications of the position.
+- Conclude with a 3 to 4 line crisp short executive takeaway highlighting the most Important implications.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Analyze {Company_Name} using the SPACE Matrix framework.
+Objective:
+Showcases company's appropriate strategic posture by evaluating on internal (Financial strength &amp; Competitive Advantage) and external dimensions (Industry Strength &amp; Environmental Stability). Categorises in Aggressive, Conservative, Defensive, or Competitive quadrants
+Instructions:
+- Use reliable publicly available information and recent business context.
+- Focus on strategic insights rather than generic statements.
+- Keep each point concise and evidence-backed.
+- Avoid unsupported speculation.
+- Follow this representation: SPACE assessment through dimensions, assessment under each dimension and score under each dimension (0-5), with final position among Aggressive, Conservative, Defensive, or Competitive quadrants.
+- Conclude with a 3 to 4 line crisp short executive takeaway highlighting the most Important implications.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Analyze {Company_Name} using the Shell Directional Policy Matrix framework.
+Objective:
+Used to evaluate a company's business based on market attractiveness and competitive capabilities. Structures company in 3x3 matrix prescribing directions like Leader, Growth, Cash Generator, Try Harder (Doubt/Quit), Custodial, Phased withdraw, Disinvest
+Instructions:
+- Use reliable publicly available information and recent business context.
+- Focus on strategic insights rather than generic statements.
+- Keep each point concise and evidence-backed.
+- Avoid unsupported speculation.
+- Follow this representation: Position of company in 3x3 matrix followed by 2-3 concise points explaining that overall and with respect to individual axis.
+- Conclude with a 3 to 4 line crisp short executive takeaway highlighting the most Important implications.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Analyze {Company_Name} using the Grand Strategy Matrix framework.
+Objective:
+Evaluates company on two factors i.e. Market Growth and Competitive Position to determine most viable long term strategies
+Instructions:
+- Use reliable publicly available information and recent business context.
+- Focus on strategic insights rather than generic statements.
+- Keep each point concise and evidence-backed.
+- Avoid unsupported speculation.
+- Follow this representation: Company in 2x2 plot with labeled axis, Strategic priority of company, Growth drivers, Biggest challenge and Outlook.
+- Conclude with a 3 to 4 line crisp short executive takeaway highlighting the most Important implications.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Analyze {Company_Name} using the Business Capability Map framework.
+Objective:
+It shows what a company does to create value, indipendent of how and who does it. Lists capabilities, Tier (Core/Strategic), Maturity and Basis
+Instructions:
+- Use reliable publicly available information and recent business context.
+- Focus on strategic insights rather than generic statements.
+- Keep each point concise and evidence-backed.
+- Avoid unsupported speculation.
+- Follow this representation: Listed capabilities, tier they belong to, maturity of each capability and a concise point under Basis as supporting proof.
+- Conclude with a 3 to 4 line crisp short executive takeaway highlighting the most Important implications.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Analyze {Company_Name} using the Operating Model Canvas framework.
+Objective:
+Used to display how a company transalate its business strategy into operational execution. It uses POLISM framework elements to uncover Processes, Organization, Locations, Informations, Suppliers, and Management Systems. 
+Instructions:
+- Use reliable publicly available information and recent business context.
+- Focus on strategic insights rather than generic statements.
+- Keep each point concise and evidence-backed.
+- Avoid unsupported speculation.
+- Follow this representation: Operating model canvas design with 6 cards for each of the POLISM elements and 2-3 concise points under each of them.
+- Conclude with a 3 to 4 line crisp short executive takeaway highlighting the most Important implications.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Analyze {Company_Name} using the Customer Value Chain framework.
+Objective:
+This shows how does the company create value throughout the customer's journey. It focuses on the end user experience. It showcases customer journey stages Discover, Analyze, Decide, Execute, and Optimize.
+Instructions:
+- Use reliable publicly available information and recent business context.
+- Focus on strategic insights rather than generic statements.
+- Keep each point concise and evidence-backed.
+- Avoid unsupported speculation.
+- Follow this representation: Contains customer journey stages, how company creates value through each stage and with what maturity..
+- Conclude with a 3 to 4 line crisp short executive takeaway highlighting the most Important implications.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Analyze {Company_Name} using the Profit Pool Analysis framework.
+Objective:
+Profit Pool analysis of shows each module/offering/product profit share with respect to revenue share
+Instructions:
+- Use reliable publicly available information and recent business context.
+- Focus on strategic insights rather than generic statements.
+- Keep each point concise and evidence-backed.
+- Avoid unsupported speculation.
+- Follow this representation: Create profit pool heat map with business segment, profit potential, company's position, and strategic priority (Expand/Scale/Invest/ Optimize/Maintain/Selective growth) for each segment of company.
+- Conclude with a 3 to 4 line crisp short executive takeaway highlighting the most Important implications.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Analyze {Company_Name} using the Revenue Model Framework framework.
+Objective:
+Executive level model show WHO pays? WHAT is paid? FOR WHAT is paid? HOW is paid? HOW MUCH is paid?
+Instructions:
+- Use reliable publicly available information and recent business context.
+- Focus on strategic insights rather than generic statements.
+- Keep each point concise and evidence-backed.
+- Avoid unsupported speculation.
+- Follow this representation: 5 cards with precise points/keywords under each card.
+- Conclude with a 3 to 4 line crisp short executive takeaway highlighting the most Important implications.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Analyze {Company_Name} using the Kotter's 8-Step Change Model framework.
+Objective:
+How successfully is the Company executing its current, most significant strategic transition across Kotter's 8 steps
+Instructions:
+- Use reliable publicly available information and recent business context.
+- Focus on strategic insights rather than generic statements.
+- Keep each point concise and evidence-backed.
+- Avoid unsupported speculation.
+- Follow this representation: cards showing company executing its trategies using kotter's 8-step model.
+- Conclude with a 3 to 4 line crisp short executive takeaway highlighting the most Important implications.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Analyze {Company_Name} using the ADKAR Model framework.
+Objective:
+Generate single static workforce evaluation for the company on pillars Awareness, Desire, Knowledge, Ability and reinforcement along with adoption status for each one of them these element throughout the employees of the company
+Instructions:
+- Use reliable publicly available information and recent business context.
+- Focus on strategic insights rather than generic statements.
+- Keep each point concise and evidence-backed.
+- Avoid unsupported speculation.
+- Follow this representation: Tabular form with 5 pillars of ADKAR, meaning of each pillar and Adoption status (High, low medium).
+- Conclude with a 3 to 4 line crisp short executive takeaway highlighting the most Important implications.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Analyze {Company_Name} using the Organizational Culture Assessment framework.
+Objective:
+Classifies the company’s internal working culture into one of four core corporate types: Clan (Collaborative), Adhocracy (Creative), Market (Competitive), or Hierarchy (Control)
+Instructions:
+- Use reliable publicly available information and recent business context.
+- Focus on strategic insights rather than generic statements.
+- Keep each point concise and evidence-backed.
+- Avoid unsupported speculation.
+- Follow this representation: Clean quadrant grid or radar chart showing which culture type dominates the company, paired with bullet points tracking internal workplace habits.
+- Conclude with a 3 to 4 line crisp short executive takeaway highlighting the most Important implications.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Analyze {Company_Name} using the Stage-Gate Model framework.
+Objective:
+This maps the formal product approval steps the company uses to move ideas from brainstorming to prototyping, testing, and public launch
+Instructions:
+- Use reliable publicly available information and recent business context.
+- Focus on strategic insights rather than generic statements.
+- Keep each point concise and evidence-backed.
+- Avoid unsupported speculation.
+- Follow this representation: Horizontal timeline diagram broken into 5 blocks (Idea, Scoping, Business Case, Development, Launch), indicating where the company commonly faces R&amp;D delays.
+- Conclude with a 3 to 4 line crisp short executive takeaway highlighting the most Important implications.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Analyze {Company_Name} using the Innovation Ambition Matrix framework.
+Objective:
+It measures the company's innovation spending across three tiers: Core improvements (optimizing old products), Adjacent moves (entering near markets), and Transformational moves (creating totally new industries)
+Instructions:
+- Use reliable publicly available information and recent business context.
+- Focus on strategic insights rather than generic statements.
+- Keep each point concise and evidence-backed.
+- Avoid unsupported speculation.
+- Follow this representation: Scatter plot with three concentric rings (Core, Adjacent, Transformational) displaying icons for the company’s active public initiatives.
+- Conclude with a 3 to 4 line crisp short executive takeaway highlighting the most Important implications.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Analyze {Company_Name} using the Disruptive Innovation Framework framework.
+Objective:
+This framework reviews whether the company's products are built for high-end markets (vulnerable to cheaper options) or low-end markets (disrupting established players)
+Instructions:
+- Use reliable publicly available information and recent business context.
+- Focus on strategic insights rather than generic statements.
+- Keep each point concise and evidence-backed.
+- Avoid unsupported speculation.
+- Follow this representation: 2-column list: Column 1 shows Disruption Vulnerabilities (threats from below); Column 2 shows Disruption Opportunities (markets the company can take over).
+- Conclude with a 3 to 4 line crisp short executive takeaway highlighting the most Important implications.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Analyze {Company_Name} using the Open Innovation Framework framework.
+Objective:
+Profiles how much the company relies on the outside world for R&amp;D, tracking things like acquisitions, open-source projects, and developer toolkits
+Instructions:
+- Use reliable publicly available information and recent business context.
+- Focus on strategic insights rather than generic statements.
+- Keep each point concise and evidence-backed.
+- Avoid unsupported speculation.
+- Follow this representation: An inside-out funnel diagram showing external inputs (e.g., buying startups) vs. internal exports (e.g., licensing code out).
+- Conclude with a 3 to 4 line crisp short executive takeaway highlighting the most Important implications.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Analyze {Company_Name} using the Innovation Radar framework.
+Objective:
+Innovation radar score with innovation dimensions Offering, Customer, Process, Platform, Network, Business Model, Brand, and Analytics with assessment of each of these dimensions as how the company is innovating on them
+Instructions:
+- Use reliable publicly available information and recent business context.
+- Focus on strategic insights rather than generic statements.
+- Keep each point concise and evidence-backed.
+- Avoid unsupported speculation.
+- Follow this representation: Tabular form with columns dimensions, assessment, innovation maturity with respective detail for all dimensions .
+- Conclude with a 3 to 4 line crisp short executive takeaway highlighting the most Important implications.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Analyze {Company_Name} using the Account Intelligence Framework framework.
+Objective:
+This gathers account-focused insights on a company (such as upcoming budget cycles, leadership changes, or current software needs) to give salespeople an edge
+Instructions:
+- Use reliable publicly available information and recent business context.
+- Focus on strategic insights rather than generic statements.
+- Keep each point concise and evidence-backed.
+- Avoid unsupported speculation.
+- Follow this representation: An executive target-card layout featuring sections like Key Decision Makers, Current Tech Friction, and Best Pitch Angles.
+- Conclude with a 3 to 4 line crisp short executive takeaway highlighting the most Important implications.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Analyze {Company_Name} using the Build vs Buy Analysis framework.
+Objective:
+Analyzes the company’s historical patterns to show if they prefer building internal proprietary tools or buying/partnering with outside platforms
+Instructions:
+- Use reliable publicly available information and recent business context.
+- Focus on strategic insights rather than generic statements.
+- Keep each point concise and evidence-backed.
+- Avoid unsupported speculation.
+- Follow this representation: Side-by-side comparison column chart charting In-house Tech Assets vs. Acquired Technical Systems.
+- Conclude with a 3 to 4 line crisp short executive takeaway highlighting the most Important implications.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Analyze {Company_Name} using the Governance and Borard composition analysis framework.
+Objective:
+This evaluates the structure, skills, and diversity of a company's directors to ensure effective oversight. It assesses independence, core competencies, and committee structures
+Instructions:
+- Use reliable publicly available information and recent business context.
+- Focus on strategic insights rather than generic statements.
+- Keep each point concise and evidence-backed.
+- Avoid unsupported speculation.
+- Follow this representation: Contains governance structure (Agency status, Governance model, Parent oversight), Leadership composition analysis, and key governance focus area.
+- Conclude with a 3 to 4 line crisp short executive takeaway highlighting the most Important implications.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Analyze {Company_Name} using the Build-Borrow-Buy Framework framework.
+Objective:
+This framework answers how should a company acquire the capability it needs to grow? It show if a company's capabilities are developed by Internal development (Build), Partnerships (borrow), acquisitions (Buy) 
+Instructions:
+- Use reliable publicly available information and recent business context.
+- Focus on strategic insights rather than generic statements.
+- Keep each point concise and evidence-backed.
+- Avoid unsupported speculation.
+- Follow this representation: Build-borrow-buy matrix snapshot with Capabilities listed in column 1, and tick mark in columns build/borrow/buy as per how company is developing them, and column 5 with recommended Approach.
+- Conclude with a 3 to 4 line crisp short executive takeaway highlighting the most Important implications.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Analyze {Company_Name} using the Technology Evolution Roadmap framework.
+Objective:
+Analyze the company's technology evolution and strategic technology direction. Identify its current technology stack and capabilities, emerging technologies it is investing in or likely to adopt, long-term technology vision, key technology focus areas
+Instructions:
+- Use reliable publicly available information and recent business context.
+- Focus on strategic insights rather than generic statements.
+- Keep each point concise and evidence-backed.
+- Avoid unsupported speculation.
+- Follow this representation: three-stage roadmap (Current → Emerging → Future), along with concise strategic insights.
+- Conclude with a 3 to 4 line crisp short executive takeaway highlighting the most Important implications.
+</t>
+  </si>
+  <si>
+    <t>Analyze {Company_Name} using SWOT Analysis.
+Objective:
+2–3 concise, crisp, evidence-backed points for quadrant: Strengths, Weaknesses, Opportunities, Threats
+Instructions:
+- Use reliable publicly available information and recent business context.
+- Focus on strategic insights rather than generic statements.
+- Keep each point concise and evidence-backed.
+- Avoid unsupported speculation.
+- Follow this representation: Four-quadrant color-coded matrix with 2-3 bullet points.
+- Conclude with a 3 to 4 line executive takeaway highlighting the most Important implications.</t>
+  </si>
+  <si>
     <t>Analyze {Company_Name} using the Business Model Canvas framework.
 Objective:
 5 key components: Value Proposition, Customer Segments, Revenue Streams, Key Partners, Channels. One concise statement for each
@@ -889,14 +1428,7 @@
 - Keep each point concise and evidence-backed.
 - Avoid unsupported speculation.
 - Follow this representation: Five-card horizontal layout with icons.
-- Conclude with a one-two line crisp short executive takeaway highlighting the most Important implications.
-- Output MUST be in GitHub Markdown.
-- DO NOT generate HTML.
-- DO NOT use &lt;table&gt;, &lt;div&gt;, or CSS.
-- Use Markdown tables.
-- Use Markdown headings.
-- Never wrap output in code fences.
-- End with Crisp short Executive Takeaway.</t>
+- Conclude with a 3 to 4 line crisp short executive takeaway highlighting the most Important implications.</t>
   </si>
   <si>
     <t>Analyze {Company_Name} using the Ansoff Matrix framework.
@@ -908,14 +1440,7 @@
 - Keep each point concise and evidence-backed.
 - Avoid unsupported speculation.
 - Follow this representation: 4 quadrant with Market vs Product.
-- Conclude with a one-two line crisp short executive takeaway highlighting the most Important implications.
-- Output MUST be in GitHub Markdown.
-- DO NOT generate HTML.
-- DO NOT use &lt;table&gt;, &lt;div&gt;, or CSS.
-- Use Markdown tables.
-- Use Markdown headings.
-- Never wrap output in code fences.
-- End with Crisp short Executive Takeaway.</t>
+- Conclude with a 3 to 4 line crisp short executive takeaway highlighting the most Important implications.</t>
   </si>
   <si>
     <t>Analyze {Company_Name} using the Porter's Five Forces framework.
@@ -927,14 +1452,7 @@
 - Keep each point concise and evidence-backed.
 - Avoid unsupported speculation.
 - Follow this representation: Horizontal rating bars for each force with overall attractiveness indicator.
-- Conclude with a one-two line crisp short executive takeaway highlighting the most Important implications.
-- Output MUST be in GitHub Markdown.
-- DO NOT generate HTML.
-- DO NOT use &lt;table&gt;, &lt;div&gt;, or CSS.
-- Use Markdown tables.
-- Use Markdown headings.
-- Never wrap output in code fences.
-- End with Crisp short Executive Takeaway.</t>
+- Conclude with a 3 to 4 line crisp short executive takeaway highlighting the most Important implications.</t>
   </si>
   <si>
     <t>Analyze {Company_Name} using the Value Chain Analysis framework.
@@ -946,14 +1464,7 @@
 - Keep each point concise and evidence-backed.
 - Avoid unsupported speculation.
 - Follow this representation: Interactive horizontal process flow with highlighted opportunity areas.
-- Conclude with a one-two line crisp short executive takeaway highlighting the most Important implications.
-- Output MUST be in GitHub Markdown.
-- DO NOT generate HTML.
-- DO NOT use &lt;table&gt;, &lt;div&gt;, or CSS.
-- Use Markdown tables.
-- Use Markdown headings.
-- Never wrap output in code fences.
-- End with Crisp short Executive Takeaway.</t>
+- Conclude with a 3 to 4 line crisp short executive takeaway highlighting the most Important implications.</t>
   </si>
   <si>
     <t>Analyze {Company_Name} using the Stakeholder Analysis framework.
@@ -965,14 +1476,7 @@
 - Keep each point concise and evidence-backed.
 - Avoid unsupported speculation.
 - Follow this representation: Structured table with influence indicators.
-- Conclude with a one-two line crisp short executive takeaway highlighting the most Important implications.
-- Output MUST be in GitHub Markdown.
-- DO NOT generate HTML.
-- DO NOT use &lt;table&gt;, &lt;div&gt;, or CSS.
-- Use Markdown tables.
-- Use Markdown headings.
-- Never wrap output in code fences.
-- End with Crisp short Executive Takeaway.</t>
+- Conclude with a 3 to 4 line crisp short executive takeaway highlighting the most Important implications.</t>
   </si>
   <si>
     <t>Analyze {Company_Name} using the Digital Maturity framework.
@@ -984,14 +1488,7 @@
 - Keep each point concise and evidence-backed.
 - Avoid unsupported speculation.
 - Follow this representation: Overall maturity badge + capability bars + technology tags.
-- Conclude with a one-two line crisp short executive takeaway highlighting the most Important implications.
-- Output MUST be in GitHub Markdown.
-- DO NOT generate HTML.
-- DO NOT use &lt;table&gt;, &lt;div&gt;, or CSS.
-- Use Markdown tables.
-- Use Markdown headings.
-- Never wrap output in code fences.
-- End with Crisp short Executive Takeaway.</t>
+- Conclude with a 3 to 4 line crisp short executive takeaway highlighting the most Important implications.</t>
   </si>
   <si>
     <t>Analyze {Company_Name} using the Opportuity Mapping framework.
@@ -1003,14 +1500,7 @@
 - Keep each point concise and evidence-backed.
 - Avoid unsupported speculation.
 - Follow this representation: Opportunity cards with Priority badges (High/Medium/Low).
-- Conclude with a one-two line crisp short executive takeaway highlighting the most Important implications.
-- Output MUST be in GitHub Markdown.
-- DO NOT generate HTML.
-- DO NOT use &lt;table&gt;, &lt;div&gt;, or CSS.
-- Use Markdown tables.
-- Use Markdown headings.
-- Never wrap output in code fences.
-- End with Crisp short Executive Takeaway.</t>
+- Conclude with a 3 to 4 line crisp short executive takeaway highlighting the most Important implications.</t>
   </si>
   <si>
     <t>Analyze {Company_Name} using the Core Competencies framework.
@@ -1022,14 +1512,7 @@
 - Keep each point concise and evidence-backed.
 - Avoid unsupported speculation.
 - Follow this representation: Cards with competency name, description and impact.
-- Conclude with a one-two line crisp short executive takeaway highlighting the most Important implications.
-- Output MUST be in GitHub Markdown.
-- DO NOT generate HTML.
-- DO NOT use &lt;table&gt;, &lt;div&gt;, or CSS.
-- Use Markdown tables.
-- Use Markdown headings.
-- Never wrap output in code fences.
-- End with Crisp short Executive Takeaway.</t>
+- Conclude with a 3 to 4 line crisp short executive takeaway highlighting the most Important implications.</t>
   </si>
   <si>
     <t>Analyze {Company_Name} using the Technology Investment Trends framework.
@@ -1041,14 +1524,7 @@
 - Keep each point concise and evidence-backed.
 - Avoid unsupported speculation.
 - Follow this representation: Technology - investment category - Investment focus (High, medium, low).
-- Conclude with a one-two line crisp short executive takeaway highlighting the most Important implications.
-- Output MUST be in GitHub Markdown.
-- DO NOT generate HTML.
-- DO NOT use &lt;table&gt;, &lt;div&gt;, or CSS.
-- Use Markdown tables.
-- Use Markdown headings.
-- Never wrap output in code fences.
-- End with Crisp short Executive Takeaway.</t>
+- Conclude with a 3 to 4 line crisp short executive takeaway highlighting the most Important implications.</t>
   </si>
   <si>
     <t>Analyze {Company_Name} using the Balanced Scorecard framework.
@@ -1060,14 +1536,7 @@
 - Keep each point concise and evidence-backed.
 - Avoid unsupported speculation.
 - Follow this representation: Status (Green/Amber/Red), 4 quadrants.
-- Conclude with a one-two line crisp short executive takeaway highlighting the most Important implications.
-- Output MUST be in GitHub Markdown.
-- DO NOT generate HTML.
-- DO NOT use &lt;table&gt;, &lt;div&gt;, or CSS.
-- Use Markdown tables.
-- Use Markdown headings.
-- Never wrap output in code fences.
-- End with Crisp short Executive Takeaway.</t>
+- Conclude with a 3 to 4 line crisp short executive takeaway highlighting the most Important implications.</t>
   </si>
   <si>
     <t>Analyze {Company_Name} using the Blue ocean strategy framework.
@@ -1079,14 +1548,7 @@
 - Keep each point concise and evidence-backed.
 - Avoid unsupported speculation.
 - Follow this representation: Blue ocean element vs evaluation table, ERRC grid.
-- Conclude with a one-two line crisp short executive takeaway highlighting the most Important implications.
-- Output MUST be in GitHub Markdown.
-- DO NOT generate HTML.
-- DO NOT use &lt;table&gt;, &lt;div&gt;, or CSS.
-- Use Markdown tables.
-- Use Markdown headings.
-- Never wrap output in code fences.
-- End with Crisp short Executive Takeaway.</t>
+- Conclude with a 3 to 4 line crisp short executive takeaway highlighting the most Important implications.</t>
   </si>
   <si>
     <t>Analyze {Company_Name} using the BCG Matrix framework.
@@ -1098,14 +1560,7 @@
 - Keep each point concise and evidence-backed.
 - Avoid unsupported speculation.
 - Follow this representation: 2x2 matrix (Stars, Cash Cows, Question Marks, Dogs).
-- Conclude with a one-two line crisp short executive takeaway highlighting the most Important implications.
-- Output MUST be in GitHub Markdown.
-- DO NOT generate HTML.
-- DO NOT use &lt;table&gt;, &lt;div&gt;, or CSS.
-- Use Markdown tables.
-- Use Markdown headings.
-- Never wrap output in code fences.
-- End with Crisp short Executive Takeaway.</t>
+- Conclude with a 3 to 4 line crisp short executive takeaway highlighting the most Important implications.</t>
   </si>
   <si>
     <t>Analyze {Company_Name} using the Gap analysis framework.
@@ -1117,17 +1572,10 @@
 - Keep each point concise and evidence-backed.
 - Avoid unsupported speculation.
 - Follow this representation: Current state - Future state - Gap - Suggestions (AI).
-- Conclude with a one-two line crisp short executive takeaway highlighting the most Important implications.
-- Output MUST be in GitHub Markdown.
-- DO NOT generate HTML.
-- DO NOT use &lt;table&gt;, &lt;div&gt;, or CSS.
-- Use Markdown tables.
-- Use Markdown headings.
-- Never wrap output in code fences.
-- End with Crisp short Executive Takeaway.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Analyze {Company_Name} using the AI adoption and Maturity framework.
+- Conclude with a 3 to 4 line crisp short executive takeaway highlighting the most Important implications.</t>
+  </si>
+  <si>
+    <t>Analyze {Company_Name} using the AI adoption and Maturity framework.
 Objective:
 AI adoption level, AI use cases, AI initiatives, governance
 Instructions:
@@ -1136,11 +1584,10 @@
 - Keep each point concise and evidence-backed.
 - Avoid unsupported speculation.
 - Follow this representation: Maturity badge, and 4 capability bar with Strategy, Data, AI, and Govrnance.
-- Conclude with a one-two line crisp short executive takeaway highlighting the most Important implications.
-</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Analyze {Company_Name} using the Value proposition canvas framework.
+- Conclude with a 3 to 4 line crisp short executive takeaway highlighting the most Important implications.</t>
+  </si>
+  <si>
+    <t>Analyze {Company_Name} using the Value proposition canvas framework.
 Objective:
 Customer needs, pain points, gains, company's value proposition
 Instructions:
@@ -1149,11 +1596,10 @@
 - Keep each point concise and evidence-backed.
 - Avoid unsupported speculation.
 - Follow this representation: Value map vs customer profile (2 columns).
-- Conclude with a one-two line crisp short executive takeaway highlighting the most Important implications.
-</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Analyze {Company_Name} using the TAM/SAM/SOM framework.
+- Conclude with a 3 to 4 line crisp short executive takeaway highlighting the most Important implications.</t>
+  </si>
+  <si>
+    <t>Analyze {Company_Name} using the TAM/SAM/SOM framework.
 Objective:
 Total addressable market, serviceable market, obtainable market
 Instructions:
@@ -1162,11 +1608,10 @@
 - Keep each point concise and evidence-backed.
 - Avoid unsupported speculation.
 - Follow this representation: Concentric circles/layered circular graph.
-- Conclude with a one-two line crisp short executive takeaway highlighting the most Important implications.
-</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Analyze {Company_Name} using the Competitor Benchmarking framework.
+- Conclude with a 3 to 4 line crisp short executive takeaway highlighting the most Important implications.</t>
+  </si>
+  <si>
+    <t>Analyze {Company_Name} using the Competitor Benchmarking framework.
 Objective:
 Company vs Top 3–5 competitors across products, technology, market presence, AI adoption
 Instructions:
@@ -1175,11 +1620,10 @@
 - Keep each point concise and evidence-backed.
 - Avoid unsupported speculation.
 - Follow this representation: Comparison table with checkmarks/ratings.
-- Conclude with a one-two line crisp short executive takeaway highlighting the most Important implications.
-</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Analyze {Company_Name} using the Competitive Landscape framework.
+- Conclude with a 3 to 4 line crisp short executive takeaway highlighting the most Important implications.</t>
+  </si>
+  <si>
+    <t>Analyze {Company_Name} using the Competitive Landscape framework.
 Objective:
 Major competitors, positioning, differentiators, market leaders, emerging players
 Instructions:
@@ -1188,11 +1632,10 @@
 - Keep each point concise and evidence-backed.
 - Avoid unsupported speculation.
 - Follow this representation: Competitor cards.
-- Conclude with a one-two line crisp short executive takeaway highlighting the most Important implications.
-</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Analyze {Company_Name} using the Market Positioning framework.
+- Conclude with a 3 to 4 line crisp short executive takeaway highlighting the most Important implications.</t>
+  </si>
+  <si>
+    <t>Analyze {Company_Name} using the Market Positioning framework.
 Objective:
 Position based on innovation, pricing, market focus, customer perception
 Instructions:
@@ -1201,11 +1644,10 @@
 - Keep each point concise and evidence-backed.
 - Avoid unsupported speculation.
 - Follow this representation: 2 Axis Positioning matrix.
-- Conclude with a one-two line crisp short executive takeaway highlighting the most Important implications.
-</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Analyze {Company_Name} using the Technology Landscape framework.
+- Conclude with a 3 to 4 line crisp short executive takeaway highlighting the most Important implications.</t>
+  </si>
+  <si>
+    <t>Analyze {Company_Name} using the Technology Landscape framework.
 Objective:
 Tech stack, cloud providers, AI platforms, Engineering tools and offerings
 Instructions:
@@ -1214,11 +1656,10 @@
 - Keep each point concise and evidence-backed.
 - Avoid unsupported speculation.
 - Follow this representation: List of offerings and products.
-- Conclude with a one-two line crisp short executive takeaway highlighting the most Important implications.
-</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Analyze {Company_Name} using the Product Portfolio Analysis framework.
+- Conclude with a 3 to 4 line crisp short executive takeaway highlighting the most Important implications.</t>
+  </si>
+  <si>
+    <t>Analyze {Company_Name} using the Product Portfolio Analysis framework.
 Objective:
 Product lines, Maturity, strategic importance
 Instructions:
@@ -1227,11 +1668,10 @@
 - Keep each point concise and evidence-backed.
 - Avoid unsupported speculation.
 - Follow this representation: Product cards by business line.
-- Conclude with a one-two line crisp short executive takeaway highlighting the most Important implications.
-</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Analyze {Company_Name} using the Product Lifecycle framework.
+- Conclude with a 3 to 4 line crisp short executive takeaway highlighting the most Important implications.</t>
+  </si>
+  <si>
+    <t>Analyze {Company_Name} using the Product Lifecycle framework.
 Objective:
 Showcase product lifecycle of key products
 Instructions:
@@ -1240,11 +1680,10 @@
 - Keep each point concise and evidence-backed.
 - Avoid unsupported speculation.
 - Follow this representation: Represent lifecycle in plot.
-- Conclude with a one-two line crisp short executive takeaway highlighting the most Important implications.
-</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Analyze {Company_Name} using the Customer Segmentation framework.
+- Conclude with a 3 to 4 line crisp short executive takeaway highlighting the most Important implications.</t>
+  </si>
+  <si>
+    <t>Analyze {Company_Name} using the Customer Segmentation framework.
 Objective:
 Customer industries, enterprise/businesses, geography, target audience
 Instructions:
@@ -1253,554 +1692,7 @@
 - Keep each point concise and evidence-backed.
 - Avoid unsupported speculation.
 - Follow this representation: segment cards.
-- Conclude with a one-two line crisp short executive takeaway highlighting the most Important implications.
-</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Analyze {Company_Name} using the ESG Assessment framework.
-Objective:
-Environmental initiatives, social responsibility, governance practices, Public ESG rating
-Instructions:
-- Use reliable publicly available information and recent business context.
-- Focus on strategic insights rather than generic statements.
-- Keep each point concise and evidence-backed.
-- Avoid unsupported speculation.
-- Follow this representation: ESG cards with Maturity status.
-- Conclude with a one-two line crisp short executive takeaway highlighting the most Important implications.
-</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Analyze {Company_Name} using the Partnership Ecosystem framework.
-Objective:
-Evaluate the company using the principles of this framework.
-Instructions:
-- Use reliable publicly available information and recent business context.
-- Focus on strategic insights rather than generic statements.
-- Keep each point concise and evidence-backed.
-- Avoid unsupported speculation.
-- Follow this representation: Executive summary.
-- Conclude with a one-two line crisp short executive takeaway highlighting the most Important implications.
-</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Analyze {Company_Name} using the Innovation Assessment framework.
-Objective:
-R&amp;D focus, patents, AI investments, innovation culture, product launches
-Instructions:
-- Use reliable publicly available information and recent business context.
-- Focus on strategic insights rather than generic statements.
-- Keep each point concise and evidence-backed.
-- Avoid unsupported speculation.
-- Follow this representation: Concise points on innovation initiatives.
-- Conclude with a one-two line crisp short executive takeaway highlighting the most Important implications.
-</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Analyze {Company_Name} using the GE-McKinsey Nine-Box Matrix framework.
-Objective:
-Business unit attractiveness vs competitive strength (high-level assessment)
-Instructions:
-- Use reliable publicly available information and recent business context.
-- Focus on strategic insights rather than generic statements.
-- Keep each point concise and evidence-backed.
-- Avoid unsupported speculation.
-- Follow this representation: 3×3 matrix with highlighted business units.
-- Conclude with a one-two line crisp short executive takeaway highlighting the most Important implications.
-</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Analyze {Company_Name} using the Strategic Partnership Opportunities framework.
-Objective:
-Highlights where company partners strategically to create competitive advantage. Contains Strategic objective, Key partnership categories, Major partners, Partnership model, Value to Company, Value to Partner, Competitive advantage created, Risk factors, and Overall Strategic Partnership Maturity
-Instructions:
-- Use reliable publicly available information and recent business context.
-- Focus on strategic insights rather than generic statements.
-- Keep each point concise and evidence-backed.
-- Avoid unsupported speculation.
-- Follow this representation: Concise pointers for each points in tabular form with partnership maturity score.
-- Conclude with a one-two line crisp short executive takeaway highlighting the most Important implications.
-</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Analyze {Company_Name} using the Sustainability Assessment framework.
-Objective:
-Overall digital maturity level, cloud adoption, AI adoption, engineering maturity, data capabilities, security posture. Tech stack details visible only for Technical Leads
-Instructions:
-- Use reliable publicly available information and recent business context.
-- Focus on strategic insights rather than generic statements.
-- Keep each point concise and evidence-backed.
-- Avoid unsupported speculation.
-- Follow this representation: Concise pointers under each of economic, innovation, etc along with overall sustainability score (out of 5).
-- Conclude with a one-two line crisp short executive takeaway highlighting the most Important implications.
-</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Analyze {Company_Name} using the McKinsey 7S framework framework.
-Objective:
-Assessment of company on 7 Elements: Strategy, Structure, system, Shared values, staff, skill and style; with a pointer on current state for each element and assessment of each pointer as Strong/average/weak
-Instructions:
-- Use reliable publicly available information and recent business context.
-- Focus on strategic insights rather than generic statements.
-- Keep each point concise and evidence-backed.
-- Avoid unsupported speculation.
-- Follow this representation: 7 cards for each elements with a concise point within each card with assessment/maturity of company on each element. With overall score.
-- Conclude with a one-two line crisp short executive takeaway highlighting the most Important implications.
-</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Analyze {Company_Name} using the Greiner Growth Model framework.
-Objective:
-Organization evolution through 6 growth phases, current position of company in 6 growth phases, status of each phases for the company, current growth challenges (3-4 key challenges and business impact)
-Instructions:
-- Use reliable publicly available information and recent business context.
-- Focus on strategic insights rather than generic statements.
-- Keep each point concise and evidence-backed.
-- Avoid unsupported speculation.
-- Follow this representation: Company position in Greiner's model curve, evolution through each phase (concise 1 sensentce on each phase) with status as Completed/Current stage/Emerging/future.
-- Conclude with a one-two line crisp short executive takeaway highlighting the most Important implications.
-</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Analyze {Company_Name} using the McKinsey's 3 Horizons of Growth framework.
-Objective:
-3 Horizon snapshot of the company including their focus, initiatives and strategic maturity. Along with horizon wise evaluation including objective, initiatives, assessment and overall 3 horizon score
-Instructions:
-- Use reliable publicly available information and recent business context.
-- Focus on strategic insights rather than generic statements.
-- Keep each point concise and evidence-backed.
-- Avoid unsupported speculation.
-- Follow this representation: 3 horizon snapshot and horizon wise evaluation , 3-4 concise pointer within each horizon and Assessment of each horizon, along with overall score.
-- Conclude with a one-two line crisp short executive takeaway highlighting the most Important implications.
-</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Analyze {Company_Name} using the TOWS Matrix framework.
-Objective:
-Putting SWOT analysis to action, combines Internal (Strength and weakness) and External (Opportunity and threats) factors to derive strategic actions/plans
-Instructions:
-- Use reliable publicly available information and recent business context.
-- Focus on strategic insights rather than generic statements.
-- Keep each point concise and evidence-backed.
-- Avoid unsupported speculation.
-- Follow this representation: 4 quadrant colour-coded matrix with 2-3 concise points in each quadrant of TOWS matrix.
-- Conclude with a one-two line crisp short executive takeaway highlighting the most Important implications.
-</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Analyze {Company_Name} using the VRIO Framework framework.
-Objective:
-Used to evaluate a company's internal resources and capabilities and its ability to sustain competitive advantage. Contains strategic resource/capability VRIO Assessment Matrix along with executive score card of each of VRIO elements
-Instructions:
-- Use reliable publicly available information and recent business context.
-- Focus on strategic insights rather than generic statements.
-- Keep each point concise and evidence-backed.
-- Avoid unsupported speculation.
-- Follow this representation: Strategic Resource/Capability assessment matrix on VRIO with competitive implications, and 4 quadrants with executive score under each of Value, Rarity, Imitability, and Organization elements.
-- Conclude with a one-two line crisp short executive takeaway highlighting the most Important implications.
-</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Analyze {Company_Name} using the Porter's Diamond Model framework.
-Objective:
-Utilized to evaluate domain or industry the company belongs to. For example, it will better evaluate insurance/healthcare domain than individual company in it
-Instructions:
-- Use reliable publicly available information and recent business context.
-- Focus on strategic insights rather than generic statements.
-- Keep each point concise and evidence-backed.
-- Avoid unsupported speculation.
-- Follow this representation: Four cards for each of the diamonds in the framework.
-- Conclude with a one-two line crisp short executive takeaway highlighting the most Important implications.
-</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Analyze {Company_Name} using the Strategic Group Mapping framework.
-Objective:
-Overall position of company, with a 2x2 strategic group map, current strategic groups, closest competitiors, key differentiators and executive insights
-Instructions:
-- Use reliable publicly available information and recent business context.
-- Focus on strategic insights rather than generic statements.
-- Keep each point concise and evidence-backed.
-- Avoid unsupported speculation.
-- Follow this representation: 1-line summary with score with a scatter plot for 2x2 map, strategic group cards with competitors, 1-line insights.
-- Conclude with a one-two line crisp short executive takeaway highlighting the most Important implications.
-</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Analyze {Company_Name} using the Bowman's Strategy Clock framework.
-Objective:
-Maps company's competitive position on 2 axes,  price vs perceived value/differentiation  - into 8 distinct positions (low price/low value, low price, hybrid, differentiation, focused differentiation, and three "doomed" high-price/low-value zones)
-Instructions:
-- Use reliable publicly available information and recent business context.
-- Focus on strategic insights rather than generic statements.
-- Keep each point concise and evidence-backed.
-- Avoid unsupported speculation.
-- Follow this representation: Price vs Perceived value chart with 8 positions.
-- Conclude with a one-two line crisp short executive takeaway highlighting the most Important implications.
-</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Analyze {Company_Name} using the Strategy Diamond framework.
-Objective:
-A strategy model that structures and challenges a company's strategic plan to make it more comprehensive and clear. Contains 5 elements Arenas, Vehicles, Differentiators, Staging and Pacing, and Economic logic
-Instructions:
-- Use reliable publicly available information and recent business context.
-- Focus on strategic insights rather than generic statements.
-- Keep each point concise and evidence-backed.
-- Avoid unsupported speculation.
-- Follow this representation: 5 cards for each element arranged in diamond shape or + shape.
-- Conclude with a one-two line crisp short executive takeaway highlighting the most Important implications.
-</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Analyze {Company_Name} using the Three C's Framework (Company, Customer, Competitor) framework.
-Objective:
-Concise line under each of  Company, Customer, Competitor, Competitive edge, and Strategic insight with respect to the company
-Instructions:
-- Use reliable publicly available information and recent business context.
-- Focus on strategic insights rather than generic statements.
-- Keep each point concise and evidence-backed.
-- Avoid unsupported speculation.
-- Follow this representation: 5 cards placed in a triagular shape with Company, customers and competitor at its edge, two card with Competitive edge and Strategic insight below them.
-- Conclude with a one-two line crisp short executive takeaway highlighting the most Important implications.
-</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Analyze {Company_Name} using the VMOST Framework framework.
-Objective:
-It showcases if a company's Vision, Mission, Objectives, Strategy, and Tactics are aligned to execute its long-term business goals. It shows concise view of strategic direction and execution maturity
-Instructions:
-- Use reliable publicly available information and recent business context.
-- Focus on strategic insights rather than generic statements.
-- Keep each point concise and evidence-backed.
-- Avoid unsupported speculation.
-- Follow this representation: VMOST snapshot with 5 components, 1 line assessment of each component and Overall alignment towards its vission and mission.
-- Conclude with a one-two line crisp short executive takeaway highlighting the most Important implications.
-</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Analyze {Company_Name} using the SOAR Analysis framework.
-Objective:
-Showcases company's strengths, opportunities, aspirations and results (performance metrics) and how well is it performing
-Instructions:
-- Use reliable publicly available information and recent business context.
-- Focus on strategic insights rather than generic statements.
-- Keep each point concise and evidence-backed.
-- Avoid unsupported speculation.
-- Follow this representation: 4 cards with concise line under each of Strengths, opportunities, aspirations and results.
-- Conclude with a one-two line crisp short executive takeaway highlighting the most Important implications.
-</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Analyze {Company_Name} using the NOISE Analysis framework.
-Objective:
-It evaluates company on 5 core elements i.e. needs, opportunities, improvements, strengths, and exceptions. It provides comprehensive business overview and helps create solution oriented action plan
-Instructions:
-- Use reliable publicly available information and recent business context.
-- Focus on strategic insights rather than generic statements.
-- Keep each point concise and evidence-backed.
-- Avoid unsupported speculation.
-- Follow this representation: Executive summary along with 5 cards for core elements Needs, opportunity, improvments, strengths and exceptions with  performance in each of them.
-- Conclude with a one-two line crisp short executive takeaway highlighting the most Important implications.
-</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Analyze {Company_Name} using the ADL Matrix framework.
-Objective:
-Evaluate company on Industry maturity stage (Embryonic, Growth, Mature, and Aging) and Competitive position (Dominant, Strong, Favorable, Tenable, and Weak)
-Instructions:
-- Use reliable publicly available information and recent business context.
-- Focus on strategic insights rather than generic statements.
-- Keep each point concise and evidence-backed.
-- Avoid unsupported speculation.
-- Follow this representation: Company position in 4x5 matrix of Industry Maturity vs Competitve position, explanation why at certain Industry maturity and competitve position backed with evidence and strategic implications of the position.
-- Conclude with a one-two line crisp short executive takeaway highlighting the most Important implications.
-</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Analyze {Company_Name} using the SPACE Matrix framework.
-Objective:
-Showcases company's appropriate strategic posture by evaluating on internal (Financial strength &amp; Competitive Advantage) and external dimensions (Industry Strength &amp; Environmental Stability). Categorises in Aggressive, Conservative, Defensive, or Competitive quadrants
-Instructions:
-- Use reliable publicly available information and recent business context.
-- Focus on strategic insights rather than generic statements.
-- Keep each point concise and evidence-backed.
-- Avoid unsupported speculation.
-- Follow this representation: SPACE assessment through dimensions, assessment under each dimension and score under each dimension (0-5), with final position among Aggressive, Conservative, Defensive, or Competitive quadrants.
-- Conclude with a one-two line crisp short executive takeaway highlighting the most Important implications.
-</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Analyze {Company_Name} using the Shell Directional Policy Matrix framework.
-Objective:
-Used to evaluate a company's business based on market attractiveness and competitive capabilities. Structures company in 3x3 matrix prescribing directions like Leader, Growth, Cash Generator, Try Harder (Doubt/Quit), Custodial, Phased withdraw, Disinvest
-Instructions:
-- Use reliable publicly available information and recent business context.
-- Focus on strategic insights rather than generic statements.
-- Keep each point concise and evidence-backed.
-- Avoid unsupported speculation.
-- Follow this representation: Position of company in 3x3 matrix followed by 2-3 concise points explaining that overall and with respect to individual axis.
-- Conclude with a one-two line crisp short executive takeaway highlighting the most Important implications.
-</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Analyze {Company_Name} using the Grand Strategy Matrix framework.
-Objective:
-Evaluates company on two factors i.e. Market Growth and Competitive Position to determine most viable long term strategies
-Instructions:
-- Use reliable publicly available information and recent business context.
-- Focus on strategic insights rather than generic statements.
-- Keep each point concise and evidence-backed.
-- Avoid unsupported speculation.
-- Follow this representation: Company in 2x2 plot with labeled axis, Strategic priority of company, Growth drivers, Biggest challenge and Outlook.
-- Conclude with a one-two line crisp short executive takeaway highlighting the most Important implications.
-</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Analyze {Company_Name} using the Business Capability Map framework.
-Objective:
-It shows what a company does to create value, indipendent of how and who does it. Lists capabilities, Tier (Core/Strategic), Maturity and Basis
-Instructions:
-- Use reliable publicly available information and recent business context.
-- Focus on strategic insights rather than generic statements.
-- Keep each point concise and evidence-backed.
-- Avoid unsupported speculation.
-- Follow this representation: Listed capabilities, tier they belong to, maturity of each capability and a concise point under Basis as supporting proof.
-- Conclude with a one-two line crisp short executive takeaway highlighting the most Important implications.
-</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Analyze {Company_Name} using the Operating Model Canvas framework.
-Objective:
-Used to display how a company transalate its business strategy into operational execution. It uses POLISM framework elements to uncover Processes, Organization, Locations, Informations, Suppliers, and Management Systems. 
-Instructions:
-- Use reliable publicly available information and recent business context.
-- Focus on strategic insights rather than generic statements.
-- Keep each point concise and evidence-backed.
-- Avoid unsupported speculation.
-- Follow this representation: Operating model canvas design with 6 cards for each of the POLISM elements and 2-3 concise points under each of them.
-- Conclude with a one-two line crisp short executive takeaway highlighting the most Important implications.
-</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Analyze {Company_Name} using the Customer Value Chain framework.
-Objective:
-This shows how does the company create value throughout the customer's journey. It focuses on the end user experience. It showcases customer journey stages Discover, Analyze, Decide, Execute, and Optimize.
-Instructions:
-- Use reliable publicly available information and recent business context.
-- Focus on strategic insights rather than generic statements.
-- Keep each point concise and evidence-backed.
-- Avoid unsupported speculation.
-- Follow this representation: Contains customer journey stages, how company creates value through each stage and with what maturity..
-- Conclude with a one-two line crisp short executive takeaway highlighting the most Important implications.
-</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Analyze {Company_Name} using the Profit Pool Analysis framework.
-Objective:
-Profit Pool analysis of shows each module/offering/product profit share with respect to revenue share
-Instructions:
-- Use reliable publicly available information and recent business context.
-- Focus on strategic insights rather than generic statements.
-- Keep each point concise and evidence-backed.
-- Avoid unsupported speculation.
-- Follow this representation: Create profit pool heat map with business segment, profit potential, company's position, and strategic priority (Expand/Scale/Invest/ Optimize/Maintain/Selective growth) for each segment of company.
-- Conclude with a one-two line crisp short executive takeaway highlighting the most Important implications.
-</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Analyze {Company_Name} using the Revenue Model Framework framework.
-Objective:
-Executive level model show WHO pays? WHAT is paid? FOR WHAT is paid? HOW is paid? HOW MUCH is paid?
-Instructions:
-- Use reliable publicly available information and recent business context.
-- Focus on strategic insights rather than generic statements.
-- Keep each point concise and evidence-backed.
-- Avoid unsupported speculation.
-- Follow this representation: 5 cards with precise points/keywords under each card.
-- Conclude with a one-two line crisp short executive takeaway highlighting the most Important implications.
-</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Analyze {Company_Name} using the Kotter's 8-Step Change Model framework.
-Objective:
-How successfully is the Company executing its current, most significant strategic transition across Kotter's 8 steps
-Instructions:
-- Use reliable publicly available information and recent business context.
-- Focus on strategic insights rather than generic statements.
-- Keep each point concise and evidence-backed.
-- Avoid unsupported speculation.
-- Follow this representation: cards showing company executing its trategies using kotter's 8-step model.
-- Conclude with a one-two line crisp short executive takeaway highlighting the most Important implications.
-</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Analyze {Company_Name} using the ADKAR Model framework.
-Objective:
-Generate single static workforce evaluation for the company on pillars Awareness, Desire, Knowledge, Ability and reinforcement along with adoption status for each one of them these element throughout the employees of the company
-Instructions:
-- Use reliable publicly available information and recent business context.
-- Focus on strategic insights rather than generic statements.
-- Keep each point concise and evidence-backed.
-- Avoid unsupported speculation.
-- Follow this representation: Tabular form with 5 pillars of ADKAR, meaning of each pillar and Adoption status (High, low medium).
-- Conclude with a one-two line crisp short executive takeaway highlighting the most Important implications.
-</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Analyze {Company_Name} using the Organizational Culture Assessment framework.
-Objective:
-Classifies the company’s internal working culture into one of four core corporate types: Clan (Collaborative), Adhocracy (Creative), Market (Competitive), or Hierarchy (Control)
-Instructions:
-- Use reliable publicly available information and recent business context.
-- Focus on strategic insights rather than generic statements.
-- Keep each point concise and evidence-backed.
-- Avoid unsupported speculation.
-- Follow this representation: Clean quadrant grid or radar chart showing which culture type dominates the company, paired with bullet points tracking internal workplace habits.
-- Conclude with a one-two line crisp short executive takeaway highlighting the most Important implications.
-</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Analyze {Company_Name} using the Stage-Gate Model framework.
-Objective:
-This maps the formal product approval steps the company uses to move ideas from brainstorming to prototyping, testing, and public launch
-Instructions:
-- Use reliable publicly available information and recent business context.
-- Focus on strategic insights rather than generic statements.
-- Keep each point concise and evidence-backed.
-- Avoid unsupported speculation.
-- Follow this representation: Horizontal timeline diagram broken into 5 blocks (Idea, Scoping, Business Case, Development, Launch), indicating where the company commonly faces R&amp;D delays.
-- Conclude with a one-two line crisp short executive takeaway highlighting the most Important implications.
-</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Analyze {Company_Name} using the Innovation Ambition Matrix framework.
-Objective:
-It measures the company's innovation spending across three tiers: Core improvements (optimizing old products), Adjacent moves (entering near markets), and Transformational moves (creating totally new industries)
-Instructions:
-- Use reliable publicly available information and recent business context.
-- Focus on strategic insights rather than generic statements.
-- Keep each point concise and evidence-backed.
-- Avoid unsupported speculation.
-- Follow this representation: Scatter plot with three concentric rings (Core, Adjacent, Transformational) displaying icons for the company’s active public initiatives.
-- Conclude with a one-two line crisp short executive takeaway highlighting the most Important implications.
-</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Analyze {Company_Name} using the Disruptive Innovation Framework framework.
-Objective:
-This framework reviews whether the company's products are built for high-end markets (vulnerable to cheaper options) or low-end markets (disrupting established players)
-Instructions:
-- Use reliable publicly available information and recent business context.
-- Focus on strategic insights rather than generic statements.
-- Keep each point concise and evidence-backed.
-- Avoid unsupported speculation.
-- Follow this representation: 2-column list: Column 1 shows Disruption Vulnerabilities (threats from below); Column 2 shows Disruption Opportunities (markets the company can take over).
-- Conclude with a one-two line crisp short executive takeaway highlighting the most Important implications.
-</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Analyze {Company_Name} using the Open Innovation Framework framework.
-Objective:
-Profiles how much the company relies on the outside world for R&amp;D, tracking things like acquisitions, open-source projects, and developer toolkits
-Instructions:
-- Use reliable publicly available information and recent business context.
-- Focus on strategic insights rather than generic statements.
-- Keep each point concise and evidence-backed.
-- Avoid unsupported speculation.
-- Follow this representation: An inside-out funnel diagram showing external inputs (e.g., buying startups) vs. internal exports (e.g., licensing code out).
-- Conclude with a one-two line crisp short executive takeaway highlighting the most Important implications.
-</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Analyze {Company_Name} using the Innovation Radar framework.
-Objective:
-Innovation radar score with innovation dimensions Offering, Customer, Process, Platform, Network, Business Model, Brand, and Analytics with assessment of each of these dimensions as how the company is innovating on them
-Instructions:
-- Use reliable publicly available information and recent business context.
-- Focus on strategic insights rather than generic statements.
-- Keep each point concise and evidence-backed.
-- Avoid unsupported speculation.
-- Follow this representation: Tabular form with columns dimensions, assessment, innovation maturity with respective detail for all dimensions .
-- Conclude with a one-two line crisp short executive takeaway highlighting the most Important implications.
-</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Analyze {Company_Name} using the Account Intelligence Framework framework.
-Objective:
-This gathers account-focused insights on a company (such as upcoming budget cycles, leadership changes, or current software needs) to give salespeople an edge
-Instructions:
-- Use reliable publicly available information and recent business context.
-- Focus on strategic insights rather than generic statements.
-- Keep each point concise and evidence-backed.
-- Avoid unsupported speculation.
-- Follow this representation: An executive target-card layout featuring sections like Key Decision Makers, Current Tech Friction, and Best Pitch Angles.
-- Conclude with a one-two line crisp short executive takeaway highlighting the most Important implications.
-</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Analyze {Company_Name} using the Build vs Buy Analysis framework.
-Objective:
-Analyzes the company’s historical patterns to show if they prefer building internal proprietary tools or buying/partnering with outside platforms
-Instructions:
-- Use reliable publicly available information and recent business context.
-- Focus on strategic insights rather than generic statements.
-- Keep each point concise and evidence-backed.
-- Avoid unsupported speculation.
-- Follow this representation: Side-by-side comparison column chart charting In-house Tech Assets vs. Acquired Technical Systems.
-- Conclude with a one-two line crisp short executive takeaway highlighting the most Important implications.
-</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Analyze {Company_Name} using the Governance and Borard composition analysis framework.
-Objective:
-This evaluates the structure, skills, and diversity of a company's directors to ensure effective oversight. It assesses independence, core competencies, and committee structures
-Instructions:
-- Use reliable publicly available information and recent business context.
-- Focus on strategic insights rather than generic statements.
-- Keep each point concise and evidence-backed.
-- Avoid unsupported speculation.
-- Follow this representation: Contains governance structure (Agency status, Governance model, Parent oversight), Leadership composition analysis, and key governance focus area.
-- Conclude with a one-two line crisp short executive takeaway highlighting the most Important implications.
-</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Analyze {Company_Name} using the Build-Borrow-Buy Framework framework.
-Objective:
-This framework answers how should a company acquire the capability it needs to grow? It show if a company's capabilities are developed by Internal development (Build), Partnerships (borrow), acquisitions (Buy) 
-Instructions:
-- Use reliable publicly available information and recent business context.
-- Focus on strategic insights rather than generic statements.
-- Keep each point concise and evidence-backed.
-- Avoid unsupported speculation.
-- Follow this representation: Build-borrow-buy matrix snapshot with Capabilities listed in column 1, and tick mark in columns build/borrow/buy as per how company is developing them, and column 5 with recommended Approach.
-- Conclude with a one-two line crisp short executive takeaway highlighting the most Important implications.
-</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Analyze {Company_Name} using the Technology Evolution Roadmap framework.
-Objective:
-Analyze the company's technology evolution and strategic technology direction. Identify its current technology stack and capabilities, emerging technologies it is investing in or likely to adopt, long-term technology vision, key technology focus areas
-Instructions:
-- Use reliable publicly available information and recent business context.
-- Focus on strategic insights rather than generic statements.
-- Keep each point concise and evidence-backed.
-- Avoid unsupported speculation.
-- Follow this representation: three-stage roadmap (Current → Emerging → Future), along with concise strategic insights.
-- Conclude with a one-two line crisp short executive takeaway highlighting the most Important implications.
-</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Analyze {Company_Name} using the Hoshin Kanri framework.
-Objective:
-Framework shows strategy deployment, how a company's vision cascades into execution and how execution feeds back into continuous improvement.
-Instructions:
-- Use reliable publicly available information and recent business context.
-- Focus on strategic insights rather than generic statements.
-- Keep each point concise and evidence-backed.
-- Avoid unsupported speculation.
-- Follow this representation: Hoshin Kanri Strategy Cascade with True north, Breakthrough Goals, Annual priorities, Strategic initiatives, KPIs, and Review.
-- Conclude with a one-two line crisp short executive takeaway highlighting the most Important implications.
-</t>
+- Conclude with a 3 to 4 line crisp short executive takeaway highlighting the most Important implications.</t>
   </si>
 </sst>
 </file>
@@ -2246,7 +2138,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:5" ht="288" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:5" ht="172.8" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>4</v>
       </c>
@@ -2260,10 +2152,10 @@
         <v>6</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>273</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" ht="302.39999999999998" x14ac:dyDescent="0.3">
+        <v>316</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" ht="288" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>7</v>
       </c>
@@ -2277,10 +2169,10 @@
         <v>10</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>274</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" ht="302.39999999999998" x14ac:dyDescent="0.3">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" ht="187.2" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
         <v>11</v>
       </c>
@@ -2294,10 +2186,10 @@
         <v>14</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>275</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" ht="288" x14ac:dyDescent="0.3">
+        <v>317</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" ht="172.8" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
         <v>15</v>
       </c>
@@ -2311,10 +2203,10 @@
         <v>18</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>276</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" ht="302.39999999999998" x14ac:dyDescent="0.3">
+        <v>318</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" ht="187.2" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
         <v>19</v>
       </c>
@@ -2328,10 +2220,10 @@
         <v>21</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>277</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" ht="302.39999999999998" x14ac:dyDescent="0.3">
+        <v>319</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" ht="187.2" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
         <v>22</v>
       </c>
@@ -2345,10 +2237,10 @@
         <v>25</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>278</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" ht="302.39999999999998" x14ac:dyDescent="0.3">
+        <v>320</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" ht="187.2" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
         <v>26</v>
       </c>
@@ -2362,10 +2254,10 @@
         <v>29</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>279</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" ht="302.39999999999998" x14ac:dyDescent="0.3">
+        <v>321</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" ht="187.2" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
         <v>30</v>
       </c>
@@ -2379,10 +2271,10 @@
         <v>33</v>
       </c>
       <c r="E9" s="4" t="s">
-        <v>280</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" ht="302.39999999999998" x14ac:dyDescent="0.3">
+        <v>322</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" ht="187.2" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
         <v>34</v>
       </c>
@@ -2396,10 +2288,10 @@
         <v>37</v>
       </c>
       <c r="E10" s="4" t="s">
-        <v>281</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" ht="288" x14ac:dyDescent="0.3">
+        <v>323</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" ht="172.8" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
         <v>38</v>
       </c>
@@ -2413,10 +2305,10 @@
         <v>41</v>
       </c>
       <c r="E11" s="4" t="s">
-        <v>282</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" ht="288" x14ac:dyDescent="0.3">
+        <v>324</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" ht="172.8" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
         <v>42</v>
       </c>
@@ -2430,10 +2322,10 @@
         <v>45</v>
       </c>
       <c r="E12" s="4" t="s">
-        <v>283</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" ht="288" x14ac:dyDescent="0.3">
+        <v>325</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" ht="172.8" x14ac:dyDescent="0.3">
       <c r="A13" s="2" t="s">
         <v>46</v>
       </c>
@@ -2447,10 +2339,10 @@
         <v>49</v>
       </c>
       <c r="E13" s="4" t="s">
-        <v>284</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" ht="302.39999999999998" x14ac:dyDescent="0.3">
+        <v>326</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" ht="187.2" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
         <v>50</v>
       </c>
@@ -2464,10 +2356,10 @@
         <v>53</v>
       </c>
       <c r="E14" s="4" t="s">
-        <v>285</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5" ht="288" x14ac:dyDescent="0.3">
+        <v>327</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" ht="172.8" x14ac:dyDescent="0.3">
       <c r="A15" s="2" t="s">
         <v>54</v>
       </c>
@@ -2481,10 +2373,10 @@
         <v>57</v>
       </c>
       <c r="E15" s="4" t="s">
-        <v>286</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5" ht="288" x14ac:dyDescent="0.3">
+        <v>328</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" ht="172.8" x14ac:dyDescent="0.3">
       <c r="A16" s="2" t="s">
         <v>58</v>
       </c>
@@ -2498,10 +2390,10 @@
         <v>61</v>
       </c>
       <c r="E16" s="4" t="s">
-        <v>287</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
+        <v>329</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" ht="172.8" x14ac:dyDescent="0.3">
       <c r="A17" s="2" t="s">
         <v>62</v>
       </c>
@@ -2515,10 +2407,10 @@
         <v>65</v>
       </c>
       <c r="E17" s="4" t="s">
-        <v>288</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" ht="172.8" x14ac:dyDescent="0.3">
       <c r="A18" s="2" t="s">
         <v>66</v>
       </c>
@@ -2532,10 +2424,10 @@
         <v>69</v>
       </c>
       <c r="E18" s="4" t="s">
-        <v>289</v>
-      </c>
-    </row>
-    <row r="19" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" ht="172.8" x14ac:dyDescent="0.3">
       <c r="A19" s="2" t="s">
         <v>70</v>
       </c>
@@ -2549,10 +2441,10 @@
         <v>73</v>
       </c>
       <c r="E19" s="4" t="s">
-        <v>290</v>
-      </c>
-    </row>
-    <row r="20" spans="1:5" ht="72" x14ac:dyDescent="0.3">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" ht="172.8" x14ac:dyDescent="0.3">
       <c r="A20" s="2" t="s">
         <v>74</v>
       </c>
@@ -2566,10 +2458,10 @@
         <v>77</v>
       </c>
       <c r="E20" s="4" t="s">
-        <v>291</v>
-      </c>
-    </row>
-    <row r="21" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
+        <v>333</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" ht="172.8" x14ac:dyDescent="0.3">
       <c r="A21" s="2" t="s">
         <v>78</v>
       </c>
@@ -2583,10 +2475,10 @@
         <v>81</v>
       </c>
       <c r="E21" s="4" t="s">
-        <v>292</v>
-      </c>
-    </row>
-    <row r="22" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" ht="172.8" x14ac:dyDescent="0.3">
       <c r="A22" s="2" t="s">
         <v>82</v>
       </c>
@@ -2600,10 +2492,10 @@
         <v>85</v>
       </c>
       <c r="E22" s="4" t="s">
-        <v>293</v>
-      </c>
-    </row>
-    <row r="23" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" ht="172.8" x14ac:dyDescent="0.3">
       <c r="A23" s="2" t="s">
         <v>86</v>
       </c>
@@ -2617,10 +2509,10 @@
         <v>89</v>
       </c>
       <c r="E23" s="4" t="s">
-        <v>294</v>
-      </c>
-    </row>
-    <row r="24" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
+        <v>336</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" ht="172.8" x14ac:dyDescent="0.3">
       <c r="A24" s="2" t="s">
         <v>90</v>
       </c>
@@ -2634,10 +2526,10 @@
         <v>93</v>
       </c>
       <c r="E24" s="4" t="s">
-        <v>295</v>
-      </c>
-    </row>
-    <row r="25" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" ht="172.8" x14ac:dyDescent="0.3">
       <c r="A25" s="2" t="s">
         <v>94</v>
       </c>
@@ -2651,10 +2543,10 @@
         <v>97</v>
       </c>
       <c r="E25" s="4" t="s">
-        <v>296</v>
-      </c>
-    </row>
-    <row r="26" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
+        <v>338</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" ht="172.8" x14ac:dyDescent="0.3">
       <c r="A26" s="2" t="s">
         <v>98</v>
       </c>
@@ -2668,7 +2560,7 @@
         <v>101</v>
       </c>
       <c r="E26" s="4" t="s">
-        <v>297</v>
+        <v>339</v>
       </c>
     </row>
     <row r="27" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
@@ -2685,7 +2577,7 @@
         <v>105</v>
       </c>
       <c r="E27" s="4" t="s">
-        <v>298</v>
+        <v>274</v>
       </c>
     </row>
     <row r="28" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
@@ -2702,7 +2594,7 @@
         <v>109</v>
       </c>
       <c r="E28" s="4" t="s">
-        <v>299</v>
+        <v>275</v>
       </c>
     </row>
     <row r="29" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
@@ -2719,10 +2611,10 @@
         <v>113</v>
       </c>
       <c r="E29" s="4" t="s">
-        <v>300</v>
-      </c>
-    </row>
-    <row r="30" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" ht="201.6" x14ac:dyDescent="0.3">
       <c r="A30" s="2" t="s">
         <v>114</v>
       </c>
@@ -2736,7 +2628,7 @@
         <v>117</v>
       </c>
       <c r="E30" s="4" t="s">
-        <v>301</v>
+        <v>277</v>
       </c>
     </row>
     <row r="31" spans="1:5" ht="115.2" x14ac:dyDescent="0.3">
@@ -2753,7 +2645,7 @@
         <v>121</v>
       </c>
       <c r="E31" s="4" t="s">
-        <v>302</v>
+        <v>278</v>
       </c>
     </row>
     <row r="32" spans="1:5" ht="72" x14ac:dyDescent="0.3">
@@ -2770,7 +2662,7 @@
         <v>125</v>
       </c>
       <c r="E32" s="4" t="s">
-        <v>303</v>
+        <v>279</v>
       </c>
     </row>
     <row r="33" spans="1:5" ht="86.4" x14ac:dyDescent="0.3">
@@ -2787,7 +2679,7 @@
         <v>129</v>
       </c>
       <c r="E33" s="4" t="s">
-        <v>304</v>
+        <v>280</v>
       </c>
     </row>
     <row r="34" spans="1:5" ht="86.4" x14ac:dyDescent="0.3">
@@ -2804,7 +2696,7 @@
         <v>133</v>
       </c>
       <c r="E34" s="4" t="s">
-        <v>305</v>
+        <v>281</v>
       </c>
     </row>
     <row r="35" spans="1:5" ht="230.4" x14ac:dyDescent="0.3">
@@ -2821,7 +2713,7 @@
         <v>137</v>
       </c>
       <c r="E35" s="4" t="s">
-        <v>339</v>
+        <v>282</v>
       </c>
     </row>
     <row r="36" spans="1:5" ht="86.4" x14ac:dyDescent="0.3">
@@ -2838,7 +2730,7 @@
         <v>141</v>
       </c>
       <c r="E36" s="4" t="s">
-        <v>306</v>
+        <v>283</v>
       </c>
     </row>
     <row r="37" spans="1:5" ht="72" x14ac:dyDescent="0.3">
@@ -2855,7 +2747,7 @@
         <v>145</v>
       </c>
       <c r="E37" s="4" t="s">
-        <v>307</v>
+        <v>284</v>
       </c>
     </row>
     <row r="38" spans="1:5" ht="86.4" x14ac:dyDescent="0.3">
@@ -2872,10 +2764,10 @@
         <v>149</v>
       </c>
       <c r="E38" s="4" t="s">
-        <v>308</v>
-      </c>
-    </row>
-    <row r="39" spans="1:5" ht="72" x14ac:dyDescent="0.3">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" ht="216" x14ac:dyDescent="0.3">
       <c r="A39" s="2" t="s">
         <v>150</v>
       </c>
@@ -2889,10 +2781,10 @@
         <v>153</v>
       </c>
       <c r="E39" s="4" t="s">
-        <v>309</v>
-      </c>
-    </row>
-    <row r="40" spans="1:5" ht="72" x14ac:dyDescent="0.3">
+        <v>286</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" ht="230.4" x14ac:dyDescent="0.3">
       <c r="A40" s="2" t="s">
         <v>154</v>
       </c>
@@ -2906,10 +2798,10 @@
         <v>157</v>
       </c>
       <c r="E40" s="4" t="s">
-        <v>310</v>
-      </c>
-    </row>
-    <row r="41" spans="1:5" ht="100.8" x14ac:dyDescent="0.3">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" ht="230.4" x14ac:dyDescent="0.3">
       <c r="A41" s="2" t="s">
         <v>158</v>
       </c>
@@ -2923,10 +2815,10 @@
         <v>161</v>
       </c>
       <c r="E41" s="4" t="s">
-        <v>311</v>
-      </c>
-    </row>
-    <row r="42" spans="1:5" ht="86.4" x14ac:dyDescent="0.3">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5" ht="230.4" x14ac:dyDescent="0.3">
       <c r="A42" s="2" t="s">
         <v>162</v>
       </c>
@@ -2940,10 +2832,10 @@
         <v>165</v>
       </c>
       <c r="E42" s="4" t="s">
-        <v>312</v>
-      </c>
-    </row>
-    <row r="43" spans="1:5" ht="72" x14ac:dyDescent="0.3">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5" ht="230.4" x14ac:dyDescent="0.3">
       <c r="A43" s="2" t="s">
         <v>166</v>
       </c>
@@ -2957,10 +2849,10 @@
         <v>169</v>
       </c>
       <c r="E43" s="4" t="s">
-        <v>313</v>
-      </c>
-    </row>
-    <row r="44" spans="1:5" ht="86.4" x14ac:dyDescent="0.3">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5" ht="230.4" x14ac:dyDescent="0.3">
       <c r="A44" s="2" t="s">
         <v>170</v>
       </c>
@@ -2974,10 +2866,10 @@
         <v>173</v>
       </c>
       <c r="E44" s="4" t="s">
-        <v>314</v>
-      </c>
-    </row>
-    <row r="45" spans="1:5" ht="72" x14ac:dyDescent="0.3">
+        <v>291</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5" ht="230.4" x14ac:dyDescent="0.3">
       <c r="A45" s="2" t="s">
         <v>174</v>
       </c>
@@ -2991,10 +2883,10 @@
         <v>177</v>
       </c>
       <c r="E45" s="4" t="s">
-        <v>315</v>
-      </c>
-    </row>
-    <row r="46" spans="1:5" ht="86.4" x14ac:dyDescent="0.3">
+        <v>292</v>
+      </c>
+    </row>
+    <row r="46" spans="1:5" ht="230.4" x14ac:dyDescent="0.3">
       <c r="A46" s="2" t="s">
         <v>178</v>
       </c>
@@ -3008,10 +2900,10 @@
         <v>181</v>
       </c>
       <c r="E46" s="4" t="s">
-        <v>316</v>
-      </c>
-    </row>
-    <row r="47" spans="1:5" ht="72" x14ac:dyDescent="0.3">
+        <v>293</v>
+      </c>
+    </row>
+    <row r="47" spans="1:5" ht="244.8" x14ac:dyDescent="0.3">
       <c r="A47" s="2" t="s">
         <v>182</v>
       </c>
@@ -3025,10 +2917,10 @@
         <v>185</v>
       </c>
       <c r="E47" s="4" t="s">
-        <v>317</v>
-      </c>
-    </row>
-    <row r="48" spans="1:5" ht="100.8" x14ac:dyDescent="0.3">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="48" spans="1:5" ht="259.2" x14ac:dyDescent="0.3">
       <c r="A48" s="2" t="s">
         <v>186</v>
       </c>
@@ -3042,10 +2934,10 @@
         <v>189</v>
       </c>
       <c r="E48" s="4" t="s">
-        <v>318</v>
-      </c>
-    </row>
-    <row r="49" spans="1:5" ht="100.8" x14ac:dyDescent="0.3">
+        <v>295</v>
+      </c>
+    </row>
+    <row r="49" spans="1:5" ht="244.8" x14ac:dyDescent="0.3">
       <c r="A49" s="2" t="s">
         <v>190</v>
       </c>
@@ -3059,10 +2951,10 @@
         <v>193</v>
       </c>
       <c r="E49" s="4" t="s">
-        <v>319</v>
-      </c>
-    </row>
-    <row r="50" spans="1:5" ht="72" x14ac:dyDescent="0.3">
+        <v>296</v>
+      </c>
+    </row>
+    <row r="50" spans="1:5" ht="230.4" x14ac:dyDescent="0.3">
       <c r="A50" s="2" t="s">
         <v>194</v>
       </c>
@@ -3076,10 +2968,10 @@
         <v>197</v>
       </c>
       <c r="E50" s="4" t="s">
-        <v>320</v>
-      </c>
-    </row>
-    <row r="51" spans="1:5" ht="72" x14ac:dyDescent="0.3">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="51" spans="1:5" ht="230.4" x14ac:dyDescent="0.3">
       <c r="A51" s="2" t="s">
         <v>198</v>
       </c>
@@ -3093,10 +2985,10 @@
         <v>201</v>
       </c>
       <c r="E51" s="4" t="s">
-        <v>321</v>
-      </c>
-    </row>
-    <row r="52" spans="1:5" ht="86.4" x14ac:dyDescent="0.3">
+        <v>298</v>
+      </c>
+    </row>
+    <row r="52" spans="1:5" ht="244.8" x14ac:dyDescent="0.3">
       <c r="A52" s="2" t="s">
         <v>202</v>
       </c>
@@ -3110,10 +3002,10 @@
         <v>205</v>
       </c>
       <c r="E52" s="4" t="s">
-        <v>322</v>
-      </c>
-    </row>
-    <row r="53" spans="1:5" ht="86.4" x14ac:dyDescent="0.3">
+        <v>299</v>
+      </c>
+    </row>
+    <row r="53" spans="1:5" ht="244.8" x14ac:dyDescent="0.3">
       <c r="A53" s="2" t="s">
         <v>206</v>
       </c>
@@ -3127,10 +3019,10 @@
         <v>209</v>
       </c>
       <c r="E53" s="4" t="s">
-        <v>323</v>
-      </c>
-    </row>
-    <row r="54" spans="1:5" ht="72" x14ac:dyDescent="0.3">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="54" spans="1:5" ht="230.4" x14ac:dyDescent="0.3">
       <c r="A54" s="2" t="s">
         <v>210</v>
       </c>
@@ -3144,10 +3036,10 @@
         <v>213</v>
       </c>
       <c r="E54" s="4" t="s">
-        <v>324</v>
-      </c>
-    </row>
-    <row r="55" spans="1:5" ht="72" x14ac:dyDescent="0.3">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="55" spans="1:5" ht="216" x14ac:dyDescent="0.3">
       <c r="A55" s="2" t="s">
         <v>214</v>
       </c>
@@ -3161,10 +3053,10 @@
         <v>217</v>
       </c>
       <c r="E55" s="4" t="s">
-        <v>325</v>
-      </c>
-    </row>
-    <row r="56" spans="1:5" ht="72" x14ac:dyDescent="0.3">
+        <v>302</v>
+      </c>
+    </row>
+    <row r="56" spans="1:5" ht="216" x14ac:dyDescent="0.3">
       <c r="A56" s="2" t="s">
         <v>218</v>
       </c>
@@ -3178,10 +3070,10 @@
         <v>221</v>
       </c>
       <c r="E56" s="4" t="s">
-        <v>326</v>
-      </c>
-    </row>
-    <row r="57" spans="1:5" ht="86.4" x14ac:dyDescent="0.3">
+        <v>303</v>
+      </c>
+    </row>
+    <row r="57" spans="1:5" ht="244.8" x14ac:dyDescent="0.3">
       <c r="A57" s="2" t="s">
         <v>222</v>
       </c>
@@ -3195,10 +3087,10 @@
         <v>225</v>
       </c>
       <c r="E57" s="4" t="s">
-        <v>327</v>
-      </c>
-    </row>
-    <row r="58" spans="1:5" ht="86.4" x14ac:dyDescent="0.3">
+        <v>304</v>
+      </c>
+    </row>
+    <row r="58" spans="1:5" ht="230.4" x14ac:dyDescent="0.3">
       <c r="A58" s="2" t="s">
         <v>226</v>
       </c>
@@ -3212,10 +3104,10 @@
         <v>229</v>
       </c>
       <c r="E58" s="4" t="s">
-        <v>328</v>
-      </c>
-    </row>
-    <row r="59" spans="1:5" ht="72" x14ac:dyDescent="0.3">
+        <v>305</v>
+      </c>
+    </row>
+    <row r="59" spans="1:5" ht="230.4" x14ac:dyDescent="0.3">
       <c r="A59" s="2" t="s">
         <v>230</v>
       </c>
@@ -3229,10 +3121,10 @@
         <v>233</v>
       </c>
       <c r="E59" s="4" t="s">
-        <v>329</v>
-      </c>
-    </row>
-    <row r="60" spans="1:5" ht="86.4" x14ac:dyDescent="0.3">
+        <v>306</v>
+      </c>
+    </row>
+    <row r="60" spans="1:5" ht="244.8" x14ac:dyDescent="0.3">
       <c r="A60" s="2" t="s">
         <v>234</v>
       </c>
@@ -3246,10 +3138,10 @@
         <v>237</v>
       </c>
       <c r="E60" s="4" t="s">
-        <v>330</v>
-      </c>
-    </row>
-    <row r="61" spans="1:5" ht="86.4" x14ac:dyDescent="0.3">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="61" spans="1:5" ht="230.4" x14ac:dyDescent="0.3">
       <c r="A61" s="2" t="s">
         <v>238</v>
       </c>
@@ -3263,10 +3155,10 @@
         <v>241</v>
       </c>
       <c r="E61" s="4" t="s">
-        <v>331</v>
-      </c>
-    </row>
-    <row r="62" spans="1:5" ht="72" x14ac:dyDescent="0.3">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="62" spans="1:5" ht="230.4" x14ac:dyDescent="0.3">
       <c r="A62" s="2" t="s">
         <v>242</v>
       </c>
@@ -3280,10 +3172,10 @@
         <v>245</v>
       </c>
       <c r="E62" s="4" t="s">
-        <v>332</v>
-      </c>
-    </row>
-    <row r="63" spans="1:5" ht="86.4" x14ac:dyDescent="0.3">
+        <v>309</v>
+      </c>
+    </row>
+    <row r="63" spans="1:5" ht="244.8" x14ac:dyDescent="0.3">
       <c r="A63" s="2" t="s">
         <v>246</v>
       </c>
@@ -3297,10 +3189,10 @@
         <v>249</v>
       </c>
       <c r="E63" s="4" t="s">
-        <v>333</v>
-      </c>
-    </row>
-    <row r="64" spans="1:5" ht="86.4" x14ac:dyDescent="0.3">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="64" spans="1:5" ht="230.4" x14ac:dyDescent="0.3">
       <c r="A64" s="2" t="s">
         <v>250</v>
       </c>
@@ -3314,10 +3206,10 @@
         <v>253</v>
       </c>
       <c r="E64" s="4" t="s">
-        <v>334</v>
-      </c>
-    </row>
-    <row r="65" spans="1:5" ht="72" x14ac:dyDescent="0.3">
+        <v>311</v>
+      </c>
+    </row>
+    <row r="65" spans="1:5" ht="230.4" x14ac:dyDescent="0.3">
       <c r="A65" s="2" t="s">
         <v>254</v>
       </c>
@@ -3331,10 +3223,10 @@
         <v>257</v>
       </c>
       <c r="E65" s="4" t="s">
-        <v>335</v>
-      </c>
-    </row>
-    <row r="66" spans="1:5" ht="86.4" x14ac:dyDescent="0.3">
+        <v>312</v>
+      </c>
+    </row>
+    <row r="66" spans="1:5" ht="230.4" x14ac:dyDescent="0.3">
       <c r="A66" s="2" t="s">
         <v>258</v>
       </c>
@@ -3348,10 +3240,10 @@
         <v>261</v>
       </c>
       <c r="E66" s="4" t="s">
-        <v>336</v>
-      </c>
-    </row>
-    <row r="67" spans="1:5" ht="86.4" x14ac:dyDescent="0.3">
+        <v>313</v>
+      </c>
+    </row>
+    <row r="67" spans="1:5" ht="259.2" x14ac:dyDescent="0.3">
       <c r="A67" s="2" t="s">
         <v>262</v>
       </c>
@@ -3365,10 +3257,10 @@
         <v>265</v>
       </c>
       <c r="E67" s="4" t="s">
-        <v>337</v>
-      </c>
-    </row>
-    <row r="68" spans="1:5" ht="100.8" x14ac:dyDescent="0.3">
+        <v>314</v>
+      </c>
+    </row>
+    <row r="68" spans="1:5" ht="244.8" x14ac:dyDescent="0.3">
       <c r="A68" s="2" t="s">
         <v>266</v>
       </c>
@@ -3382,7 +3274,7 @@
         <v>269</v>
       </c>
       <c r="E68" s="4" t="s">
-        <v>338</v>
+        <v>315</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Codebase cleanup and refactoring
</commit_message>
<xml_diff>
--- a/config/Framework_Intelligence.xlsx
+++ b/config/Framework_Intelligence.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Shubham.baranwal\Downloads\Company_Report_Generator\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{481A9BF5-BDDB-4273-97B5-B72E54F5391B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3AE8E342-6114-4B2D-886A-18577BADBC47}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -523,9 +523,6 @@
     <t>F43</t>
   </si>
   <si>
-    <t>Three C's Framework (Company, Customer, Competitor)</t>
-  </si>
-  <si>
     <t>Analyze the company using the Three C's Framework (Company, Customer, Competitor) framework. Concise line under each of  Company, Customer, Competitor, Competitive edge, and Strategic insight with respect to the company Focus on strategic, evidence-backed insights derived from public information. Keep the analysis concise, executive-ready, and actionable.</t>
   </si>
   <si>
@@ -797,9 +794,6 @@
   </si>
   <si>
     <t>F83</t>
-  </si>
-  <si>
-    <t>Governance and Borard composition analysis</t>
   </si>
   <si>
     <t>Analyze the company using the Governance and Borard composition analysis framework. This evaluates the structure, skills, and diversity of a company's directors to ensure effective oversight. It assesses independence, core competencies, and committee structures Focus on strategic, evidence-backed insights derived from public information. Keep the analysis concise, executive-ready, and actionable.</t>
@@ -1693,6 +1687,12 @@
 - Avoid unsupported speculation.
 - Follow this representation: segment cards.
 - Conclude with a 3 to 4 line crisp short executive takeaway highlighting the most Important implications.</t>
+  </si>
+  <si>
+    <t>3 C's Framework (Company, Customer, Competitor)</t>
+  </si>
+  <si>
+    <t>Governance and Board composition analysis</t>
   </si>
 </sst>
 </file>
@@ -2126,7 +2126,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="C1" s="6" t="s">
         <v>1</v>
@@ -2146,13 +2146,13 @@
         <v>5</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="D2" s="4" t="s">
         <v>6</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>316</v>
+        <v>314</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="288" x14ac:dyDescent="0.3">
@@ -2169,7 +2169,7 @@
         <v>10</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="187.2" x14ac:dyDescent="0.3">
@@ -2186,7 +2186,7 @@
         <v>14</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>317</v>
+        <v>315</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="172.8" x14ac:dyDescent="0.3">
@@ -2203,7 +2203,7 @@
         <v>18</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>318</v>
+        <v>316</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="187.2" x14ac:dyDescent="0.3">
@@ -2214,13 +2214,13 @@
         <v>20</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
       <c r="D6" s="4" t="s">
         <v>21</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>319</v>
+        <v>317</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="187.2" x14ac:dyDescent="0.3">
@@ -2237,7 +2237,7 @@
         <v>25</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>320</v>
+        <v>318</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="187.2" x14ac:dyDescent="0.3">
@@ -2254,7 +2254,7 @@
         <v>29</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>321</v>
+        <v>319</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="187.2" x14ac:dyDescent="0.3">
@@ -2271,7 +2271,7 @@
         <v>33</v>
       </c>
       <c r="E9" s="4" t="s">
-        <v>322</v>
+        <v>320</v>
       </c>
     </row>
     <row r="10" spans="1:5" ht="187.2" x14ac:dyDescent="0.3">
@@ -2288,7 +2288,7 @@
         <v>37</v>
       </c>
       <c r="E10" s="4" t="s">
-        <v>323</v>
+        <v>321</v>
       </c>
     </row>
     <row r="11" spans="1:5" ht="172.8" x14ac:dyDescent="0.3">
@@ -2305,7 +2305,7 @@
         <v>41</v>
       </c>
       <c r="E11" s="4" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
     </row>
     <row r="12" spans="1:5" ht="172.8" x14ac:dyDescent="0.3">
@@ -2322,7 +2322,7 @@
         <v>45</v>
       </c>
       <c r="E12" s="4" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
     </row>
     <row r="13" spans="1:5" ht="172.8" x14ac:dyDescent="0.3">
@@ -2339,7 +2339,7 @@
         <v>49</v>
       </c>
       <c r="E13" s="4" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
     </row>
     <row r="14" spans="1:5" ht="187.2" x14ac:dyDescent="0.3">
@@ -2356,7 +2356,7 @@
         <v>53</v>
       </c>
       <c r="E14" s="4" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
     </row>
     <row r="15" spans="1:5" ht="172.8" x14ac:dyDescent="0.3">
@@ -2373,7 +2373,7 @@
         <v>57</v>
       </c>
       <c r="E15" s="4" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
     </row>
     <row r="16" spans="1:5" ht="172.8" x14ac:dyDescent="0.3">
@@ -2390,7 +2390,7 @@
         <v>61</v>
       </c>
       <c r="E16" s="4" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
     </row>
     <row r="17" spans="1:5" ht="172.8" x14ac:dyDescent="0.3">
@@ -2407,7 +2407,7 @@
         <v>65</v>
       </c>
       <c r="E17" s="4" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
     </row>
     <row r="18" spans="1:5" ht="172.8" x14ac:dyDescent="0.3">
@@ -2424,7 +2424,7 @@
         <v>69</v>
       </c>
       <c r="E18" s="4" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
     </row>
     <row r="19" spans="1:5" ht="172.8" x14ac:dyDescent="0.3">
@@ -2441,7 +2441,7 @@
         <v>73</v>
       </c>
       <c r="E19" s="4" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
     </row>
     <row r="20" spans="1:5" ht="172.8" x14ac:dyDescent="0.3">
@@ -2458,7 +2458,7 @@
         <v>77</v>
       </c>
       <c r="E20" s="4" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
     </row>
     <row r="21" spans="1:5" ht="172.8" x14ac:dyDescent="0.3">
@@ -2475,7 +2475,7 @@
         <v>81</v>
       </c>
       <c r="E21" s="4" t="s">
-        <v>334</v>
+        <v>332</v>
       </c>
     </row>
     <row r="22" spans="1:5" ht="172.8" x14ac:dyDescent="0.3">
@@ -2492,7 +2492,7 @@
         <v>85</v>
       </c>
       <c r="E22" s="4" t="s">
-        <v>335</v>
+        <v>333</v>
       </c>
     </row>
     <row r="23" spans="1:5" ht="172.8" x14ac:dyDescent="0.3">
@@ -2509,7 +2509,7 @@
         <v>89</v>
       </c>
       <c r="E23" s="4" t="s">
-        <v>336</v>
+        <v>334</v>
       </c>
     </row>
     <row r="24" spans="1:5" ht="172.8" x14ac:dyDescent="0.3">
@@ -2526,7 +2526,7 @@
         <v>93</v>
       </c>
       <c r="E24" s="4" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
     </row>
     <row r="25" spans="1:5" ht="172.8" x14ac:dyDescent="0.3">
@@ -2543,7 +2543,7 @@
         <v>97</v>
       </c>
       <c r="E25" s="4" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
     </row>
     <row r="26" spans="1:5" ht="172.8" x14ac:dyDescent="0.3">
@@ -2560,7 +2560,7 @@
         <v>101</v>
       </c>
       <c r="E26" s="4" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
     </row>
     <row r="27" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
@@ -2577,7 +2577,7 @@
         <v>105</v>
       </c>
       <c r="E27" s="4" t="s">
-        <v>274</v>
+        <v>272</v>
       </c>
     </row>
     <row r="28" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
@@ -2594,10 +2594,10 @@
         <v>109</v>
       </c>
       <c r="E28" s="4" t="s">
-        <v>275</v>
-      </c>
-    </row>
-    <row r="29" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" ht="187.2" x14ac:dyDescent="0.3">
       <c r="A29" s="2" t="s">
         <v>110</v>
       </c>
@@ -2611,10 +2611,10 @@
         <v>113</v>
       </c>
       <c r="E29" s="4" t="s">
-        <v>276</v>
-      </c>
-    </row>
-    <row r="30" spans="1:5" ht="201.6" x14ac:dyDescent="0.3">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" ht="187.2" x14ac:dyDescent="0.3">
       <c r="A30" s="2" t="s">
         <v>114</v>
       </c>
@@ -2628,10 +2628,10 @@
         <v>117</v>
       </c>
       <c r="E30" s="4" t="s">
-        <v>277</v>
-      </c>
-    </row>
-    <row r="31" spans="1:5" ht="115.2" x14ac:dyDescent="0.3">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" ht="230.4" x14ac:dyDescent="0.3">
       <c r="A31" s="2" t="s">
         <v>118</v>
       </c>
@@ -2645,10 +2645,10 @@
         <v>121</v>
       </c>
       <c r="E31" s="4" t="s">
-        <v>278</v>
-      </c>
-    </row>
-    <row r="32" spans="1:5" ht="72" x14ac:dyDescent="0.3">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" ht="216" x14ac:dyDescent="0.3">
       <c r="A32" s="2" t="s">
         <v>122</v>
       </c>
@@ -2662,10 +2662,10 @@
         <v>125</v>
       </c>
       <c r="E32" s="4" t="s">
-        <v>279</v>
-      </c>
-    </row>
-    <row r="33" spans="1:5" ht="86.4" x14ac:dyDescent="0.3">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" ht="216" x14ac:dyDescent="0.3">
       <c r="A33" s="2" t="s">
         <v>126</v>
       </c>
@@ -2679,10 +2679,10 @@
         <v>129</v>
       </c>
       <c r="E33" s="4" t="s">
-        <v>280</v>
-      </c>
-    </row>
-    <row r="34" spans="1:5" ht="86.4" x14ac:dyDescent="0.3">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" ht="216" x14ac:dyDescent="0.3">
       <c r="A34" s="2" t="s">
         <v>130</v>
       </c>
@@ -2696,10 +2696,10 @@
         <v>133</v>
       </c>
       <c r="E34" s="4" t="s">
-        <v>281</v>
-      </c>
-    </row>
-    <row r="35" spans="1:5" ht="230.4" x14ac:dyDescent="0.3">
+        <v>279</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" ht="216" x14ac:dyDescent="0.3">
       <c r="A35" s="2" t="s">
         <v>134</v>
       </c>
@@ -2713,10 +2713,10 @@
         <v>137</v>
       </c>
       <c r="E35" s="4" t="s">
-        <v>282</v>
-      </c>
-    </row>
-    <row r="36" spans="1:5" ht="86.4" x14ac:dyDescent="0.3">
+        <v>280</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" ht="216" x14ac:dyDescent="0.3">
       <c r="A36" s="2" t="s">
         <v>138</v>
       </c>
@@ -2730,10 +2730,10 @@
         <v>141</v>
       </c>
       <c r="E36" s="4" t="s">
-        <v>283</v>
-      </c>
-    </row>
-    <row r="37" spans="1:5" ht="72" x14ac:dyDescent="0.3">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" ht="216" x14ac:dyDescent="0.3">
       <c r="A37" s="2" t="s">
         <v>142</v>
       </c>
@@ -2747,10 +2747,10 @@
         <v>145</v>
       </c>
       <c r="E37" s="4" t="s">
-        <v>284</v>
-      </c>
-    </row>
-    <row r="38" spans="1:5" ht="86.4" x14ac:dyDescent="0.3">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" ht="244.8" x14ac:dyDescent="0.3">
       <c r="A38" s="2" t="s">
         <v>146</v>
       </c>
@@ -2764,10 +2764,10 @@
         <v>149</v>
       </c>
       <c r="E38" s="4" t="s">
-        <v>285</v>
-      </c>
-    </row>
-    <row r="39" spans="1:5" ht="216" x14ac:dyDescent="0.3">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" ht="201.6" x14ac:dyDescent="0.3">
       <c r="A39" s="2" t="s">
         <v>150</v>
       </c>
@@ -2781,10 +2781,10 @@
         <v>153</v>
       </c>
       <c r="E39" s="4" t="s">
-        <v>286</v>
-      </c>
-    </row>
-    <row r="40" spans="1:5" ht="230.4" x14ac:dyDescent="0.3">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" ht="216" x14ac:dyDescent="0.3">
       <c r="A40" s="2" t="s">
         <v>154</v>
       </c>
@@ -2798,10 +2798,10 @@
         <v>157</v>
       </c>
       <c r="E40" s="4" t="s">
-        <v>287</v>
-      </c>
-    </row>
-    <row r="41" spans="1:5" ht="230.4" x14ac:dyDescent="0.3">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" ht="216" x14ac:dyDescent="0.3">
       <c r="A41" s="2" t="s">
         <v>158</v>
       </c>
@@ -2815,10 +2815,10 @@
         <v>161</v>
       </c>
       <c r="E41" s="4" t="s">
-        <v>288</v>
-      </c>
-    </row>
-    <row r="42" spans="1:5" ht="230.4" x14ac:dyDescent="0.3">
+        <v>286</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5" ht="216" x14ac:dyDescent="0.3">
       <c r="A42" s="2" t="s">
         <v>162</v>
       </c>
@@ -2832,449 +2832,449 @@
         <v>165</v>
       </c>
       <c r="E42" s="4" t="s">
-        <v>289</v>
-      </c>
-    </row>
-    <row r="43" spans="1:5" ht="230.4" x14ac:dyDescent="0.3">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5" ht="216" x14ac:dyDescent="0.3">
       <c r="A43" s="2" t="s">
         <v>166</v>
       </c>
       <c r="B43" s="2" t="s">
+        <v>338</v>
+      </c>
+      <c r="C43" s="4" t="s">
         <v>167</v>
       </c>
-      <c r="C43" s="4" t="s">
+      <c r="D43" s="4" t="s">
         <v>168</v>
       </c>
-      <c r="D43" s="4" t="s">
+      <c r="E43" s="4" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5" ht="216" x14ac:dyDescent="0.3">
+      <c r="A44" s="2" t="s">
         <v>169</v>
       </c>
-      <c r="E43" s="4" t="s">
+      <c r="B44" s="2" t="s">
+        <v>170</v>
+      </c>
+      <c r="C44" s="4" t="s">
+        <v>171</v>
+      </c>
+      <c r="D44" s="4" t="s">
+        <v>172</v>
+      </c>
+      <c r="E44" s="4" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5" ht="216" x14ac:dyDescent="0.3">
+      <c r="A45" s="2" t="s">
+        <v>173</v>
+      </c>
+      <c r="B45" s="2" t="s">
+        <v>174</v>
+      </c>
+      <c r="C45" s="4" t="s">
+        <v>175</v>
+      </c>
+      <c r="D45" s="4" t="s">
+        <v>176</v>
+      </c>
+      <c r="E45" s="4" t="s">
         <v>290</v>
       </c>
     </row>
-    <row r="44" spans="1:5" ht="230.4" x14ac:dyDescent="0.3">
-      <c r="A44" s="2" t="s">
-        <v>170</v>
-      </c>
-      <c r="B44" s="2" t="s">
-        <v>171</v>
-      </c>
-      <c r="C44" s="4" t="s">
-        <v>172</v>
-      </c>
-      <c r="D44" s="4" t="s">
-        <v>173</v>
-      </c>
-      <c r="E44" s="4" t="s">
+    <row r="46" spans="1:5" ht="216" x14ac:dyDescent="0.3">
+      <c r="A46" s="2" t="s">
+        <v>177</v>
+      </c>
+      <c r="B46" s="2" t="s">
+        <v>178</v>
+      </c>
+      <c r="C46" s="4" t="s">
+        <v>179</v>
+      </c>
+      <c r="D46" s="4" t="s">
+        <v>180</v>
+      </c>
+      <c r="E46" s="4" t="s">
         <v>291</v>
       </c>
     </row>
-    <row r="45" spans="1:5" ht="230.4" x14ac:dyDescent="0.3">
-      <c r="A45" s="2" t="s">
-        <v>174</v>
-      </c>
-      <c r="B45" s="2" t="s">
-        <v>175</v>
-      </c>
-      <c r="C45" s="4" t="s">
-        <v>176</v>
-      </c>
-      <c r="D45" s="4" t="s">
-        <v>177</v>
-      </c>
-      <c r="E45" s="4" t="s">
+    <row r="47" spans="1:5" ht="230.4" x14ac:dyDescent="0.3">
+      <c r="A47" s="2" t="s">
+        <v>181</v>
+      </c>
+      <c r="B47" s="2" t="s">
+        <v>182</v>
+      </c>
+      <c r="C47" s="4" t="s">
+        <v>183</v>
+      </c>
+      <c r="D47" s="4" t="s">
+        <v>184</v>
+      </c>
+      <c r="E47" s="4" t="s">
         <v>292</v>
       </c>
     </row>
-    <row r="46" spans="1:5" ht="230.4" x14ac:dyDescent="0.3">
-      <c r="A46" s="2" t="s">
-        <v>178</v>
-      </c>
-      <c r="B46" s="2" t="s">
-        <v>179</v>
-      </c>
-      <c r="C46" s="4" t="s">
-        <v>180</v>
-      </c>
-      <c r="D46" s="4" t="s">
-        <v>181</v>
-      </c>
-      <c r="E46" s="4" t="s">
+    <row r="48" spans="1:5" ht="244.8" x14ac:dyDescent="0.3">
+      <c r="A48" s="2" t="s">
+        <v>185</v>
+      </c>
+      <c r="B48" s="2" t="s">
+        <v>186</v>
+      </c>
+      <c r="C48" s="4" t="s">
+        <v>187</v>
+      </c>
+      <c r="D48" s="4" t="s">
+        <v>188</v>
+      </c>
+      <c r="E48" s="4" t="s">
         <v>293</v>
       </c>
     </row>
-    <row r="47" spans="1:5" ht="244.8" x14ac:dyDescent="0.3">
-      <c r="A47" s="2" t="s">
-        <v>182</v>
-      </c>
-      <c r="B47" s="2" t="s">
-        <v>183</v>
-      </c>
-      <c r="C47" s="4" t="s">
-        <v>184</v>
-      </c>
-      <c r="D47" s="4" t="s">
-        <v>185</v>
-      </c>
-      <c r="E47" s="4" t="s">
+    <row r="49" spans="1:5" ht="230.4" x14ac:dyDescent="0.3">
+      <c r="A49" s="2" t="s">
+        <v>189</v>
+      </c>
+      <c r="B49" s="2" t="s">
+        <v>190</v>
+      </c>
+      <c r="C49" s="4" t="s">
+        <v>191</v>
+      </c>
+      <c r="D49" s="4" t="s">
+        <v>192</v>
+      </c>
+      <c r="E49" s="4" t="s">
         <v>294</v>
       </c>
     </row>
-    <row r="48" spans="1:5" ht="259.2" x14ac:dyDescent="0.3">
-      <c r="A48" s="2" t="s">
-        <v>186</v>
-      </c>
-      <c r="B48" s="2" t="s">
-        <v>187</v>
-      </c>
-      <c r="C48" s="4" t="s">
-        <v>188</v>
-      </c>
-      <c r="D48" s="4" t="s">
-        <v>189</v>
-      </c>
-      <c r="E48" s="4" t="s">
+    <row r="50" spans="1:5" ht="216" x14ac:dyDescent="0.3">
+      <c r="A50" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="B50" s="2" t="s">
+        <v>194</v>
+      </c>
+      <c r="C50" s="4" t="s">
+        <v>195</v>
+      </c>
+      <c r="D50" s="4" t="s">
+        <v>196</v>
+      </c>
+      <c r="E50" s="4" t="s">
         <v>295</v>
       </c>
     </row>
-    <row r="49" spans="1:5" ht="244.8" x14ac:dyDescent="0.3">
-      <c r="A49" s="2" t="s">
-        <v>190</v>
-      </c>
-      <c r="B49" s="2" t="s">
-        <v>191</v>
-      </c>
-      <c r="C49" s="4" t="s">
-        <v>192</v>
-      </c>
-      <c r="D49" s="4" t="s">
-        <v>193</v>
-      </c>
-      <c r="E49" s="4" t="s">
+    <row r="51" spans="1:5" ht="216" x14ac:dyDescent="0.3">
+      <c r="A51" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="B51" s="2" t="s">
+        <v>198</v>
+      </c>
+      <c r="C51" s="4" t="s">
+        <v>199</v>
+      </c>
+      <c r="D51" s="4" t="s">
+        <v>200</v>
+      </c>
+      <c r="E51" s="4" t="s">
         <v>296</v>
       </c>
     </row>
-    <row r="50" spans="1:5" ht="230.4" x14ac:dyDescent="0.3">
-      <c r="A50" s="2" t="s">
-        <v>194</v>
-      </c>
-      <c r="B50" s="2" t="s">
-        <v>195</v>
-      </c>
-      <c r="C50" s="4" t="s">
-        <v>196</v>
-      </c>
-      <c r="D50" s="4" t="s">
-        <v>197</v>
-      </c>
-      <c r="E50" s="4" t="s">
+    <row r="52" spans="1:5" ht="230.4" x14ac:dyDescent="0.3">
+      <c r="A52" s="2" t="s">
+        <v>201</v>
+      </c>
+      <c r="B52" s="2" t="s">
+        <v>202</v>
+      </c>
+      <c r="C52" s="4" t="s">
+        <v>203</v>
+      </c>
+      <c r="D52" s="4" t="s">
+        <v>204</v>
+      </c>
+      <c r="E52" s="4" t="s">
         <v>297</v>
       </c>
     </row>
-    <row r="51" spans="1:5" ht="230.4" x14ac:dyDescent="0.3">
-      <c r="A51" s="2" t="s">
-        <v>198</v>
-      </c>
-      <c r="B51" s="2" t="s">
-        <v>199</v>
-      </c>
-      <c r="C51" s="4" t="s">
-        <v>200</v>
-      </c>
-      <c r="D51" s="4" t="s">
-        <v>201</v>
-      </c>
-      <c r="E51" s="4" t="s">
+    <row r="53" spans="1:5" ht="230.4" x14ac:dyDescent="0.3">
+      <c r="A53" s="2" t="s">
+        <v>205</v>
+      </c>
+      <c r="B53" s="2" t="s">
+        <v>206</v>
+      </c>
+      <c r="C53" s="4" t="s">
+        <v>207</v>
+      </c>
+      <c r="D53" s="4" t="s">
+        <v>208</v>
+      </c>
+      <c r="E53" s="4" t="s">
         <v>298</v>
       </c>
     </row>
-    <row r="52" spans="1:5" ht="244.8" x14ac:dyDescent="0.3">
-      <c r="A52" s="2" t="s">
-        <v>202</v>
-      </c>
-      <c r="B52" s="2" t="s">
-        <v>203</v>
-      </c>
-      <c r="C52" s="4" t="s">
-        <v>204</v>
-      </c>
-      <c r="D52" s="4" t="s">
-        <v>205</v>
-      </c>
-      <c r="E52" s="4" t="s">
+    <row r="54" spans="1:5" ht="216" x14ac:dyDescent="0.3">
+      <c r="A54" s="2" t="s">
+        <v>209</v>
+      </c>
+      <c r="B54" s="2" t="s">
+        <v>210</v>
+      </c>
+      <c r="C54" s="4" t="s">
+        <v>211</v>
+      </c>
+      <c r="D54" s="4" t="s">
+        <v>212</v>
+      </c>
+      <c r="E54" s="4" t="s">
         <v>299</v>
       </c>
     </row>
-    <row r="53" spans="1:5" ht="244.8" x14ac:dyDescent="0.3">
-      <c r="A53" s="2" t="s">
-        <v>206</v>
-      </c>
-      <c r="B53" s="2" t="s">
-        <v>207</v>
-      </c>
-      <c r="C53" s="4" t="s">
-        <v>208</v>
-      </c>
-      <c r="D53" s="4" t="s">
-        <v>209</v>
-      </c>
-      <c r="E53" s="4" t="s">
+    <row r="55" spans="1:5" ht="201.6" x14ac:dyDescent="0.3">
+      <c r="A55" s="2" t="s">
+        <v>213</v>
+      </c>
+      <c r="B55" s="2" t="s">
+        <v>214</v>
+      </c>
+      <c r="C55" s="4" t="s">
+        <v>215</v>
+      </c>
+      <c r="D55" s="4" t="s">
+        <v>216</v>
+      </c>
+      <c r="E55" s="4" t="s">
         <v>300</v>
       </c>
     </row>
-    <row r="54" spans="1:5" ht="230.4" x14ac:dyDescent="0.3">
-      <c r="A54" s="2" t="s">
-        <v>210</v>
-      </c>
-      <c r="B54" s="2" t="s">
-        <v>211</v>
-      </c>
-      <c r="C54" s="4" t="s">
-        <v>212</v>
-      </c>
-      <c r="D54" s="4" t="s">
-        <v>213</v>
-      </c>
-      <c r="E54" s="4" t="s">
+    <row r="56" spans="1:5" ht="201.6" x14ac:dyDescent="0.3">
+      <c r="A56" s="2" t="s">
+        <v>217</v>
+      </c>
+      <c r="B56" s="2" t="s">
+        <v>218</v>
+      </c>
+      <c r="C56" s="4" t="s">
+        <v>219</v>
+      </c>
+      <c r="D56" s="4" t="s">
+        <v>220</v>
+      </c>
+      <c r="E56" s="4" t="s">
         <v>301</v>
       </c>
     </row>
-    <row r="55" spans="1:5" ht="216" x14ac:dyDescent="0.3">
-      <c r="A55" s="2" t="s">
-        <v>214</v>
-      </c>
-      <c r="B55" s="2" t="s">
-        <v>215</v>
-      </c>
-      <c r="C55" s="4" t="s">
-        <v>216</v>
-      </c>
-      <c r="D55" s="4" t="s">
-        <v>217</v>
-      </c>
-      <c r="E55" s="4" t="s">
+    <row r="57" spans="1:5" ht="230.4" x14ac:dyDescent="0.3">
+      <c r="A57" s="2" t="s">
+        <v>221</v>
+      </c>
+      <c r="B57" s="2" t="s">
+        <v>222</v>
+      </c>
+      <c r="C57" s="4" t="s">
+        <v>223</v>
+      </c>
+      <c r="D57" s="4" t="s">
+        <v>224</v>
+      </c>
+      <c r="E57" s="4" t="s">
         <v>302</v>
       </c>
     </row>
-    <row r="56" spans="1:5" ht="216" x14ac:dyDescent="0.3">
-      <c r="A56" s="2" t="s">
-        <v>218</v>
-      </c>
-      <c r="B56" s="2" t="s">
-        <v>219</v>
-      </c>
-      <c r="C56" s="4" t="s">
-        <v>220</v>
-      </c>
-      <c r="D56" s="4" t="s">
-        <v>221</v>
-      </c>
-      <c r="E56" s="4" t="s">
+    <row r="58" spans="1:5" ht="216" x14ac:dyDescent="0.3">
+      <c r="A58" s="2" t="s">
+        <v>225</v>
+      </c>
+      <c r="B58" s="2" t="s">
+        <v>226</v>
+      </c>
+      <c r="C58" s="4" t="s">
+        <v>227</v>
+      </c>
+      <c r="D58" s="4" t="s">
+        <v>228</v>
+      </c>
+      <c r="E58" s="4" t="s">
         <v>303</v>
       </c>
     </row>
-    <row r="57" spans="1:5" ht="244.8" x14ac:dyDescent="0.3">
-      <c r="A57" s="2" t="s">
-        <v>222</v>
-      </c>
-      <c r="B57" s="2" t="s">
-        <v>223</v>
-      </c>
-      <c r="C57" s="4" t="s">
-        <v>224</v>
-      </c>
-      <c r="D57" s="4" t="s">
-        <v>225</v>
-      </c>
-      <c r="E57" s="4" t="s">
+    <row r="59" spans="1:5" ht="216" x14ac:dyDescent="0.3">
+      <c r="A59" s="2" t="s">
+        <v>229</v>
+      </c>
+      <c r="B59" s="2" t="s">
+        <v>230</v>
+      </c>
+      <c r="C59" s="4" t="s">
+        <v>231</v>
+      </c>
+      <c r="D59" s="4" t="s">
+        <v>232</v>
+      </c>
+      <c r="E59" s="4" t="s">
         <v>304</v>
       </c>
     </row>
-    <row r="58" spans="1:5" ht="230.4" x14ac:dyDescent="0.3">
-      <c r="A58" s="2" t="s">
-        <v>226</v>
-      </c>
-      <c r="B58" s="2" t="s">
-        <v>227</v>
-      </c>
-      <c r="C58" s="4" t="s">
-        <v>228</v>
-      </c>
-      <c r="D58" s="4" t="s">
-        <v>229</v>
-      </c>
-      <c r="E58" s="4" t="s">
+    <row r="60" spans="1:5" ht="230.4" x14ac:dyDescent="0.3">
+      <c r="A60" s="2" t="s">
+        <v>233</v>
+      </c>
+      <c r="B60" s="2" t="s">
+        <v>234</v>
+      </c>
+      <c r="C60" s="4" t="s">
+        <v>235</v>
+      </c>
+      <c r="D60" s="4" t="s">
+        <v>236</v>
+      </c>
+      <c r="E60" s="4" t="s">
         <v>305</v>
       </c>
     </row>
-    <row r="59" spans="1:5" ht="230.4" x14ac:dyDescent="0.3">
-      <c r="A59" s="2" t="s">
-        <v>230</v>
-      </c>
-      <c r="B59" s="2" t="s">
-        <v>231</v>
-      </c>
-      <c r="C59" s="4" t="s">
-        <v>232</v>
-      </c>
-      <c r="D59" s="4" t="s">
-        <v>233</v>
-      </c>
-      <c r="E59" s="4" t="s">
+    <row r="61" spans="1:5" ht="216" x14ac:dyDescent="0.3">
+      <c r="A61" s="2" t="s">
+        <v>237</v>
+      </c>
+      <c r="B61" s="2" t="s">
+        <v>238</v>
+      </c>
+      <c r="C61" s="4" t="s">
+        <v>239</v>
+      </c>
+      <c r="D61" s="4" t="s">
+        <v>240</v>
+      </c>
+      <c r="E61" s="4" t="s">
         <v>306</v>
       </c>
     </row>
-    <row r="60" spans="1:5" ht="244.8" x14ac:dyDescent="0.3">
-      <c r="A60" s="2" t="s">
-        <v>234</v>
-      </c>
-      <c r="B60" s="2" t="s">
-        <v>235</v>
-      </c>
-      <c r="C60" s="4" t="s">
-        <v>236</v>
-      </c>
-      <c r="D60" s="4" t="s">
-        <v>237</v>
-      </c>
-      <c r="E60" s="4" t="s">
+    <row r="62" spans="1:5" ht="216" x14ac:dyDescent="0.3">
+      <c r="A62" s="2" t="s">
+        <v>241</v>
+      </c>
+      <c r="B62" s="2" t="s">
+        <v>242</v>
+      </c>
+      <c r="C62" s="4" t="s">
+        <v>243</v>
+      </c>
+      <c r="D62" s="4" t="s">
+        <v>244</v>
+      </c>
+      <c r="E62" s="4" t="s">
         <v>307</v>
       </c>
     </row>
-    <row r="61" spans="1:5" ht="230.4" x14ac:dyDescent="0.3">
-      <c r="A61" s="2" t="s">
-        <v>238</v>
-      </c>
-      <c r="B61" s="2" t="s">
-        <v>239</v>
-      </c>
-      <c r="C61" s="4" t="s">
-        <v>240</v>
-      </c>
-      <c r="D61" s="4" t="s">
-        <v>241</v>
-      </c>
-      <c r="E61" s="4" t="s">
+    <row r="63" spans="1:5" ht="230.4" x14ac:dyDescent="0.3">
+      <c r="A63" s="2" t="s">
+        <v>245</v>
+      </c>
+      <c r="B63" s="2" t="s">
+        <v>246</v>
+      </c>
+      <c r="C63" s="4" t="s">
+        <v>247</v>
+      </c>
+      <c r="D63" s="4" t="s">
+        <v>248</v>
+      </c>
+      <c r="E63" s="4" t="s">
         <v>308</v>
       </c>
     </row>
-    <row r="62" spans="1:5" ht="230.4" x14ac:dyDescent="0.3">
-      <c r="A62" s="2" t="s">
-        <v>242</v>
-      </c>
-      <c r="B62" s="2" t="s">
-        <v>243</v>
-      </c>
-      <c r="C62" s="4" t="s">
-        <v>244</v>
-      </c>
-      <c r="D62" s="4" t="s">
-        <v>245</v>
-      </c>
-      <c r="E62" s="4" t="s">
+    <row r="64" spans="1:5" ht="216" x14ac:dyDescent="0.3">
+      <c r="A64" s="2" t="s">
+        <v>249</v>
+      </c>
+      <c r="B64" s="2" t="s">
+        <v>250</v>
+      </c>
+      <c r="C64" s="4" t="s">
+        <v>251</v>
+      </c>
+      <c r="D64" s="4" t="s">
+        <v>252</v>
+      </c>
+      <c r="E64" s="4" t="s">
         <v>309</v>
       </c>
     </row>
-    <row r="63" spans="1:5" ht="244.8" x14ac:dyDescent="0.3">
-      <c r="A63" s="2" t="s">
-        <v>246</v>
-      </c>
-      <c r="B63" s="2" t="s">
-        <v>247</v>
-      </c>
-      <c r="C63" s="4" t="s">
-        <v>248</v>
-      </c>
-      <c r="D63" s="4" t="s">
-        <v>249</v>
-      </c>
-      <c r="E63" s="4" t="s">
+    <row r="65" spans="1:5" ht="216" x14ac:dyDescent="0.3">
+      <c r="A65" s="2" t="s">
+        <v>253</v>
+      </c>
+      <c r="B65" s="2" t="s">
+        <v>254</v>
+      </c>
+      <c r="C65" s="4" t="s">
+        <v>255</v>
+      </c>
+      <c r="D65" s="4" t="s">
+        <v>256</v>
+      </c>
+      <c r="E65" s="4" t="s">
         <v>310</v>
       </c>
     </row>
-    <row r="64" spans="1:5" ht="230.4" x14ac:dyDescent="0.3">
-      <c r="A64" s="2" t="s">
-        <v>250</v>
-      </c>
-      <c r="B64" s="2" t="s">
-        <v>251</v>
-      </c>
-      <c r="C64" s="4" t="s">
-        <v>252</v>
-      </c>
-      <c r="D64" s="4" t="s">
-        <v>253</v>
-      </c>
-      <c r="E64" s="4" t="s">
+    <row r="66" spans="1:5" ht="216" x14ac:dyDescent="0.3">
+      <c r="A66" s="2" t="s">
+        <v>257</v>
+      </c>
+      <c r="B66" s="2" t="s">
+        <v>339</v>
+      </c>
+      <c r="C66" s="4" t="s">
+        <v>258</v>
+      </c>
+      <c r="D66" s="4" t="s">
+        <v>259</v>
+      </c>
+      <c r="E66" s="4" t="s">
         <v>311</v>
       </c>
     </row>
-    <row r="65" spans="1:5" ht="230.4" x14ac:dyDescent="0.3">
-      <c r="A65" s="2" t="s">
-        <v>254</v>
-      </c>
-      <c r="B65" s="2" t="s">
-        <v>255</v>
-      </c>
-      <c r="C65" s="4" t="s">
-        <v>256</v>
-      </c>
-      <c r="D65" s="4" t="s">
-        <v>257</v>
-      </c>
-      <c r="E65" s="4" t="s">
+    <row r="67" spans="1:5" ht="244.8" x14ac:dyDescent="0.3">
+      <c r="A67" s="2" t="s">
+        <v>260</v>
+      </c>
+      <c r="B67" s="2" t="s">
+        <v>261</v>
+      </c>
+      <c r="C67" s="4" t="s">
+        <v>262</v>
+      </c>
+      <c r="D67" s="4" t="s">
+        <v>263</v>
+      </c>
+      <c r="E67" s="4" t="s">
         <v>312</v>
       </c>
     </row>
-    <row r="66" spans="1:5" ht="230.4" x14ac:dyDescent="0.3">
-      <c r="A66" s="2" t="s">
-        <v>258</v>
-      </c>
-      <c r="B66" s="2" t="s">
-        <v>259</v>
-      </c>
-      <c r="C66" s="4" t="s">
-        <v>260</v>
-      </c>
-      <c r="D66" s="4" t="s">
-        <v>261</v>
-      </c>
-      <c r="E66" s="4" t="s">
+    <row r="68" spans="1:5" ht="230.4" x14ac:dyDescent="0.3">
+      <c r="A68" s="2" t="s">
+        <v>264</v>
+      </c>
+      <c r="B68" s="2" t="s">
+        <v>265</v>
+      </c>
+      <c r="C68" s="4" t="s">
+        <v>266</v>
+      </c>
+      <c r="D68" s="4" t="s">
+        <v>267</v>
+      </c>
+      <c r="E68" s="4" t="s">
         <v>313</v>
-      </c>
-    </row>
-    <row r="67" spans="1:5" ht="259.2" x14ac:dyDescent="0.3">
-      <c r="A67" s="2" t="s">
-        <v>262</v>
-      </c>
-      <c r="B67" s="2" t="s">
-        <v>263</v>
-      </c>
-      <c r="C67" s="4" t="s">
-        <v>264</v>
-      </c>
-      <c r="D67" s="4" t="s">
-        <v>265</v>
-      </c>
-      <c r="E67" s="4" t="s">
-        <v>314</v>
-      </c>
-    </row>
-    <row r="68" spans="1:5" ht="244.8" x14ac:dyDescent="0.3">
-      <c r="A68" s="2" t="s">
-        <v>266</v>
-      </c>
-      <c r="B68" s="2" t="s">
-        <v>267</v>
-      </c>
-      <c r="C68" s="4" t="s">
-        <v>268</v>
-      </c>
-      <c r="D68" s="4" t="s">
-        <v>269</v>
-      </c>
-      <c r="E68" s="4" t="s">
-        <v>315</v>
       </c>
     </row>
   </sheetData>

</xml_diff>